<commit_message>
Update forecast data 2026-09-07_20-35-54
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712829226240098</v>
+        <v>4.712828362466269</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711697544571431</v>
+        <v>4.711701570027312</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720218258689325</v>
+        <v>4.72022319335514</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707005014566412</v>
+        <v>4.707015209548521</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694352517329468</v>
+        <v>4.694362828324006</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678428012096183</v>
+        <v>4.678438412701133</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673437265587149</v>
+        <v>4.673447692772864</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686513378454542</v>
+        <v>4.686523805862614</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702475552506931</v>
+        <v>4.702488103173977</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70565562155251</v>
+        <v>4.705663956232113</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694727466316546</v>
+        <v>4.694735963584399</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664760852105111</v>
+        <v>4.664770054364148</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64965478907347</v>
+        <v>4.649656247766455</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641397887793743</v>
+        <v>4.641401355753608</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636229468079178</v>
+        <v>4.636231621294042</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634000025443999</v>
+        <v>4.63400508600646</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637386774180293</v>
+        <v>4.637388029434613</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634433432788318</v>
+        <v>4.634430616425403</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627572586513217</v>
+        <v>4.627564119292262</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623830242067585</v>
+        <v>4.623821195662067</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599189969185458</v>
+        <v>4.5991810575185</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579547532084061</v>
+        <v>4.579528453249773</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560763647454222</v>
+        <v>4.560732820078613</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522738934910617</v>
+        <v>4.522693352479147</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519827795125801</v>
+        <v>4.51976300914156</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532639107427949</v>
+        <v>4.532567402298564</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551504334638937</v>
+        <v>4.551431263020852</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584016945188253</v>
+        <v>4.583934961630905</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.60268110008412</v>
+        <v>4.602576758523661</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675312210228611</v>
+        <v>4.675192490838439</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.710918737755398</v>
+        <v>4.710791765795532</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777625660608566</v>
+        <v>4.777506297458766</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81315911416908</v>
+        <v>4.813089058055148</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810913054911899</v>
+        <v>4.810844504283387</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820120289690154</v>
+        <v>4.820051847136511</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862359389817028</v>
+        <v>4.862352545698111</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855099431919156</v>
+        <v>4.855095513011761</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852933116733523</v>
+        <v>4.852965040336404</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830113792941448</v>
+        <v>4.830136717345404</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83796207761786</v>
+        <v>4.837992264350623</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.89091896975472</v>
+        <v>4.890972427987665</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917554658120146</v>
+        <v>4.917586702665563</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926773227848448</v>
+        <v>4.926805716116651</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916886302267982</v>
+        <v>4.916917784037906</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897750190874862</v>
+        <v>4.897775499986401</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896014919583529</v>
+        <v>4.89605716138086</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896624662798262</v>
+        <v>4.896683800911049</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893917575744304</v>
+        <v>4.893996247716969</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878412118205981</v>
+        <v>4.878493125547972</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855093518748941</v>
+        <v>4.855161790561401</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828857940322568</v>
+        <v>4.828923279545706</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819612975471641</v>
+        <v>4.819675334258687</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789605860621924</v>
+        <v>4.789658138615056</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761659710069396</v>
+        <v>4.761712478124496</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750749565597044</v>
+        <v>4.750802754663469</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754842867808298</v>
+        <v>4.75492603808968</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749814344484644</v>
+        <v>4.749864675630718</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750292390937112</v>
+        <v>4.75029974133819</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756268582995891</v>
+        <v>4.756218153311637</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.761944664291351</v>
+        <v>4.761814602988355</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.768560630600362</v>
+        <v>4.770281017176671</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.766262947625982</v>
+        <v>4.768354454706945</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.76389122825009</v>
+        <v>4.766182619667067</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.764357573874866</v>
+        <v>4.767180933652939</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.761886944507113</v>
+        <v>4.764947467187709</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.763875716223932</v>
+        <v>4.767079731271346</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.769604590455818</v>
+        <v>4.773033786019767</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.791818176310524</v>
+        <v>4.795412455185019</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.805605718258124</v>
+        <v>4.809666393264026</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.817977399660849</v>
+        <v>4.822558921990124</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.822561947468646</v>
+        <v>4.82755054014376</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.85112151113958</v>
+        <v>4.85497953002834</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.861080803518474</v>
+        <v>4.864876814256053</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.865269253010146</v>
+        <v>4.871235292989915</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-09_20-36-24
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712827516875114</v>
+        <v>4.712826688898511</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711705510313568</v>
+        <v>4.711709368104639</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720228024281589</v>
+        <v>4.720232754705416</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707025189679342</v>
+        <v>4.707034961678518</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694372922031895</v>
+        <v>4.694382805248683</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678448594130004</v>
+        <v>4.678458563237488</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673457900281656</v>
+        <v>4.673467894982034</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686534013747786</v>
+        <v>4.686544008968816</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702500390703306</v>
+        <v>4.702512423282033</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705672116417798</v>
+        <v>4.705680107531508</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.69474428286196</v>
+        <v>4.694752429682687</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664779063679747</v>
+        <v>4.664787886056014</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649657680223506</v>
+        <v>4.649659087125539</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641404754399376</v>
+        <v>4.641408085783102</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636233729336757</v>
+        <v>4.63623579361415</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634010041078285</v>
+        <v>4.634014893922307</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637389261370556</v>
+        <v>4.637390470619842</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63442786018221</v>
+        <v>4.634425162156351</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627555828699173</v>
+        <v>4.627547709267148</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623812338613461</v>
+        <v>4.623803665039477</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599172332969664</v>
+        <v>4.599163789710033</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579509783702753</v>
+        <v>4.579491510424674</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560702658050102</v>
+        <v>4.560673140089456</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522648748809525</v>
+        <v>4.522605092758925</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519699610650981</v>
+        <v>4.519637555622751</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532497225552421</v>
+        <v>4.532428528925222</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551359742918113</v>
+        <v>4.551289725537449</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583854709678318</v>
+        <v>4.583776135173777</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.602474584474827</v>
+        <v>4.602374511193525</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675075262070983</v>
+        <v>4.67496044712602</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.710667436246173</v>
+        <v>4.710545667597456</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777389375307209</v>
+        <v>4.777274820164163</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813020437872252</v>
+        <v>4.812953209999444</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.8107773492309</v>
+        <v>4.810711547660942</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819984785937888</v>
+        <v>4.819919064814757</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862345828905948</v>
+        <v>4.862339235977041</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855091659008873</v>
+        <v>4.855087868418163</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852996301107256</v>
+        <v>4.853026919464206</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830159152297028</v>
+        <v>4.830181113289477</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838021813670714</v>
+        <v>4.838050745529655</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891024769608165</v>
+        <v>4.891076029219022</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917618056086352</v>
+        <v>4.917648740440355</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926837507264453</v>
+        <v>4.926868623419965</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916948610742869</v>
+        <v>4.916978802560228</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897800278996381</v>
+        <v>4.897824544325708</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896098536876009</v>
+        <v>4.896139072375901</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896741746431618</v>
+        <v>4.896798534958128</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894073320654828</v>
+        <v>4.89414884269004</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878572481187556</v>
+        <v>4.878650235034792</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855228655830992</v>
+        <v>4.855294157529301</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828987246429827</v>
+        <v>4.829049883717544</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819736376926983</v>
+        <v>4.819796144671987</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789709287631924</v>
+        <v>4.789759343743658</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.76176413326494</v>
+        <v>4.76181471009892</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750854861633961</v>
+        <v>4.75090591886169</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755007635643826</v>
+        <v>4.755087703960374</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749914184907065</v>
+        <v>4.749962890820445</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750307162715842</v>
+        <v>4.750314646562812</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756168967482076</v>
+        <v>4.75612098237721</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.761687265200296</v>
+        <v>4.761562568326339</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.770088963557884</v>
+        <v>4.769900631846586</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.770315573783168</v>
+        <v>4.772077745881822</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.768386801072422</v>
+        <v>4.770347031430449</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.76928626020412</v>
+        <v>4.771100124759355</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.767222121929361</v>
+        <v>4.769101354961776</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.769226342171574</v>
+        <v>4.770926324784289</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.775236270586676</v>
+        <v>4.776920560282744</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.797569720150197</v>
+        <v>4.799107607574248</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.812053525482776</v>
+        <v>4.813676269259172</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.824927025657713</v>
+        <v>4.826387955618502</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.829956158159145</v>
+        <v>4.831079260861712</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.855808876396642</v>
+        <v>4.855081699709633</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.864696420267836</v>
+        <v>4.862409349704134</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.870060513619679</v>
+        <v>4.865548913985291</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.865664519920969</v>
+        <v>4.84960676106363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-10_20-36-28
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712826688898511</v>
+        <v>4.712825877991756</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711709368104639</v>
+        <v>4.711713145964164</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720232754705416</v>
+        <v>4.720237387730116</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707034961678518</v>
+        <v>4.707044531988419</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694382805248683</v>
+        <v>4.69439248448952</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678458563237488</v>
+        <v>4.678468326595434</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673467894982034</v>
+        <v>4.673477683459176</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686544008968816</v>
+        <v>4.686553798101733</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702512423282033</v>
+        <v>4.702524208761227</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705680107531508</v>
+        <v>4.705687934772906</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694752429682687</v>
+        <v>4.694760409353073</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664787886056014</v>
+        <v>4.664796527250543</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649659087125539</v>
+        <v>4.649660469131081</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641408085783102</v>
+        <v>4.641411351876862</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.63623579361415</v>
+        <v>4.636237815475218</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634014893922307</v>
+        <v>4.634019647668239</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637390470619842</v>
+        <v>4.637391657792126</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634425162156351</v>
+        <v>4.634422520524776</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627547709267148</v>
+        <v>4.627539755752561</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623803665039477</v>
+        <v>4.623795169298914</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599163789710033</v>
+        <v>4.599155422150178</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579491510424674</v>
+        <v>4.579473620943034</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560673140089456</v>
+        <v>4.560644245814053</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522605092758925</v>
+        <v>4.522562354490031</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519637555622751</v>
+        <v>4.51957680186637</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532428528925222</v>
+        <v>4.532361266160228</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551289725537449</v>
+        <v>4.551221164106279</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583776135173777</v>
+        <v>4.583699186190393</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.602374511193525</v>
+        <v>4.602276474644039</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.67496044712602</v>
+        <v>4.674847972323882</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.710545667597456</v>
+        <v>4.71042638165266</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777274820164163</v>
+        <v>4.777162560994952</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812953209999444</v>
+        <v>4.812887332561647</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810711547660942</v>
+        <v>4.810647059152129</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819919064814757</v>
+        <v>4.819854644111115</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862339235977041</v>
+        <v>4.862332763569821</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855087868418163</v>
+        <v>4.855084139787335</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853026919464206</v>
+        <v>4.853056914995827</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830181113289477</v>
+        <v>4.830202615169495</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838050745529655</v>
+        <v>4.838079079055971</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891076029219022</v>
+        <v>4.891126240008752</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917648740440355</v>
+        <v>4.917678776859102</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926868623419965</v>
+        <v>4.926899085787412</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916978802560228</v>
+        <v>4.917008378849467</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897824544325708</v>
+        <v>4.897848311726447</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896139072375901</v>
+        <v>4.896178793135926</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896798534958128</v>
+        <v>4.896854200690728</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.89414884269004</v>
+        <v>4.894222860047433</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878650235034792</v>
+        <v>4.878726435012799</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855294157529301</v>
+        <v>4.855358336897194</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829049883717544</v>
+        <v>4.829111232396487</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819796144671987</v>
+        <v>4.819854676989126</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789759343743658</v>
+        <v>4.789808341505299</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.76181471009892</v>
+        <v>4.761864241823671</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.75090591886169</v>
+        <v>4.750955957436474</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755087703960374</v>
+        <v>4.755166284970175</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749962890820445</v>
+        <v>4.750010811396937</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750314646562812</v>
+        <v>4.750322184948478</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.75612098237721</v>
+        <v>4.756074156763228</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.761562568326339</v>
+        <v>4.761440432993016</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.769900631846586</v>
+        <v>4.769715918050476</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.772077745881822</v>
+        <v>4.773850952700521</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.770347031430449</v>
+        <v>4.772350473225859</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.771100124759355</v>
+        <v>4.773003469246612</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.769101354961776</v>
+        <v>4.771191864740993</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.770926324784289</v>
+        <v>4.772923301354007</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.776920560282744</v>
+        <v>4.778992137160541</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.799107607574248</v>
+        <v>4.801155889698806</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.813676269259172</v>
+        <v>4.815947216455949</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.826387955618502</v>
+        <v>4.828664428271225</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.831079260861712</v>
+        <v>4.833473333731758</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.855081699709633</v>
+        <v>4.856231948583563</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.862409349704134</v>
+        <v>4.862978977482751</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.865548913985291</v>
+        <v>4.866103463352059</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.84960676106363</v>
+        <v>4.857986583016739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-11_22-19-05
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712825877991756</v>
+        <v>4.712825083632379</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711713145964164</v>
+        <v>4.711716846350654</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720237387730116</v>
+        <v>4.720241926332727</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707044531988419</v>
+        <v>4.707053906788294</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.69439248448952</v>
+        <v>4.694401966003475</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678468326595434</v>
+        <v>4.678477890507288</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673477683459176</v>
+        <v>4.673487272029384</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686553798101733</v>
+        <v>4.686563387454256</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702524208761227</v>
+        <v>4.702535754672957</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705687934772906</v>
+        <v>4.70569560313064</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694760409353073</v>
+        <v>4.694768226964147</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664796527250543</v>
+        <v>4.664804992786923</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649660469131081</v>
+        <v>4.649661826877127</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641411351876862</v>
+        <v>4.641414554576599</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636237815475218</v>
+        <v>4.636239796214078</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634019647668239</v>
+        <v>4.634024305319395</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637391657792126</v>
+        <v>4.637392823475931</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634422520524776</v>
+        <v>4.634419933539677</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627539755752561</v>
+        <v>4.627531963123705</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623795169298914</v>
+        <v>4.623786845979426</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599155422150178</v>
+        <v>4.599147224927982</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579473620943034</v>
+        <v>4.579456103302864</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560644245814053</v>
+        <v>4.560615955691214</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522562354490031</v>
+        <v>4.522520505403431</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.51957680186637</v>
+        <v>4.519517308937096</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532361266160228</v>
+        <v>4.532295392905128</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551221164106279</v>
+        <v>4.551154013769374</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583699186190393</v>
+        <v>4.583623812917766</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.602276474644039</v>
+        <v>4.602180413363245</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674847972323882</v>
+        <v>4.674737766948789</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.71042638165266</v>
+        <v>4.710309503361827</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777162560994952</v>
+        <v>4.777052529574151</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812887332561647</v>
+        <v>4.812822765343354</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810647059152129</v>
+        <v>4.810583844873182</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819854644111115</v>
+        <v>4.819791485715693</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862332763569821</v>
+        <v>4.862326408459483</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855084139787335</v>
+        <v>4.855080471703156</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853056914995827</v>
+        <v>4.853086306502794</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830202615169495</v>
+        <v>4.830223672170751</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838079079055971</v>
+        <v>4.838106832597148</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891126240008752</v>
+        <v>4.891175433823067</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917678776859102</v>
+        <v>4.917708185595806</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926899085787412</v>
+        <v>4.926928914694709</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917008378849467</v>
+        <v>4.917037358193086</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897848311726447</v>
+        <v>4.897871596315417</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896178793135926</v>
+        <v>4.896217723411807</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896854200690728</v>
+        <v>4.896908776499268</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894222860047433</v>
+        <v>4.894295417137783</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878726435012799</v>
+        <v>4.878801127155455</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855358336897194</v>
+        <v>4.855421233530969</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829111232396487</v>
+        <v>4.829171331788372</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819854676989126</v>
+        <v>4.819912011760517</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789808341505299</v>
+        <v>4.789856314034413</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761864241823671</v>
+        <v>4.761912760296189</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750955957436474</v>
+        <v>4.75100500724515</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755166284970175</v>
+        <v>4.755243419112889</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750010811396937</v>
+        <v>4.750057964192875</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750322184948478</v>
+        <v>4.750329770479683</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756074156763228</v>
+        <v>4.756028451202599</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.761440432993016</v>
+        <v>4.761320782902022</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.769715918050476</v>
+        <v>4.769534721888192</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.773850952700521</v>
+        <v>4.774494588647405</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.772350473225859</v>
+        <v>4.773018156069778</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.773003469246612</v>
+        <v>4.773356627884668</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.771191864740993</v>
+        <v>4.771115726787531</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.772923301354007</v>
+        <v>4.772716273448551</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.778992137160541</v>
+        <v>4.778519332901203</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.801155889698806</v>
+        <v>4.800121469992744</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.815947216455949</v>
+        <v>4.814447972700771</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.828664428271225</v>
+        <v>4.82648708817755</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.833473333731758</v>
+        <v>4.82985286193632</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.856231948583563</v>
+        <v>4.84978583912619</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.862978977482751</v>
+        <v>4.85323937921676</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.866103463352059</v>
+        <v>4.850668983646926</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.857986583016739</v>
+        <v>4.818941555210066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-12_09-40-55
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712825083632379</v>
+        <v>4.712824305319012</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711716846350654</v>
+        <v>4.711720471622831</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720241926332727</v>
+        <v>4.720246373370204</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707053906788294</v>
+        <v>4.707063092007568</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694401966003475</v>
+        <v>4.694411255786973</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678477890507288</v>
+        <v>4.678487261021663</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673487272029384</v>
+        <v>4.673496666753665</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686563387454256</v>
+        <v>4.686572783079335</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702535754672957</v>
+        <v>4.70254706824634</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70569560313064</v>
+        <v>4.705703117392943</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694768226964147</v>
+        <v>4.694775887402308</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664804992786923</v>
+        <v>4.664813287966525</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649661826877127</v>
+        <v>4.649663160979965</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641414554576599</v>
+        <v>4.641417695705744</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636239796214078</v>
+        <v>4.636241737072735</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634024305319395</v>
+        <v>4.634028869759001</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637392823475931</v>
+        <v>4.637393968239524</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634419933539677</v>
+        <v>4.63441739952466</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627531963123705</v>
+        <v>4.627524326550192</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623786845979426</v>
+        <v>4.623778689886046</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599147224927982</v>
+        <v>4.599139192897209</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579456103302864</v>
+        <v>4.579438946040194</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560615955691214</v>
+        <v>4.560588250994405</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522520505403431</v>
+        <v>4.522479518074154</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519517308937096</v>
+        <v>4.519459038046687</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532295392905128</v>
+        <v>4.532230866615171</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551154013769374</v>
+        <v>4.551088231491788</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583623812917766</v>
+        <v>4.583549967555488</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.602180413363245</v>
+        <v>4.60208626833289</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674737766948789</v>
+        <v>4.674629763101535</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.710309503361827</v>
+        <v>4.710194960665286</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777052529574151</v>
+        <v>4.776944660348331</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812822765343354</v>
+        <v>4.812759469707357</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810583844873182</v>
+        <v>4.810521867505683</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819791485715693</v>
+        <v>4.819729552987704</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862326408459483</v>
+        <v>4.862320167533048</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855080471703156</v>
+        <v>4.855076862790468</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853086306502794</v>
+        <v>4.85311511203709</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830223672170751</v>
+        <v>4.83024429794513</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838106832597148</v>
+        <v>4.838134023759035</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891175433823067</v>
+        <v>4.89122364123207</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917708185595806</v>
+        <v>4.917736986070422</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926928914694709</v>
+        <v>4.926958129638141</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917037358193086</v>
+        <v>4.917065758435097</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897871596315417</v>
+        <v>4.897894412605767</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896217723411807</v>
+        <v>4.896255886508449</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896908776499268</v>
+        <v>4.896962293987137</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894295417137783</v>
+        <v>4.894366556645702</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878801127155455</v>
+        <v>4.878874355699407</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855421233530969</v>
+        <v>4.855482885463426</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829171331788372</v>
+        <v>4.829230219632698</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819912011760517</v>
+        <v>4.819968185336446</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789856314034413</v>
+        <v>4.789903293084866</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761912760296189</v>
+        <v>4.761960296099769</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.75100500724515</v>
+        <v>4.75105309702856</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755243419112889</v>
+        <v>4.755319145401227</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750057964192875</v>
+        <v>4.750104366305884</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750329770479683</v>
+        <v>4.750337396264429</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756028451202599</v>
+        <v>4.75598382796027</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.761320782902022</v>
+        <v>4.76120354468628</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.769534721888192</v>
+        <v>4.769356946631756</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.774494588647405</v>
+        <v>4.775231050130876</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.773018156069778</v>
+        <v>4.773815533342352</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.773356627884668</v>
+        <v>4.773969965449256</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.771115726787531</v>
+        <v>4.771795006121531</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.772716273448551</v>
+        <v>4.77346104222134</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.778519332901203</v>
+        <v>4.779329503766722</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.800121469992744</v>
+        <v>4.80074397919816</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.814447972700771</v>
+        <v>4.814984921494941</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.82648708817755</v>
+        <v>4.826752858292267</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.82985286193632</v>
+        <v>4.829946316136876</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.84978583912619</v>
+        <v>4.848423254583714</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.85323937921676</v>
+        <v>4.850737672598219</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.850668983646926</v>
+        <v>4.846871488886876</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.818941555210066</v>
+        <v>4.815774623596267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-14_20-36-27
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712824305319012</v>
+        <v>4.712823542570339</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711720471622831</v>
+        <v>4.711724024044635</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720246373370204</v>
+        <v>4.720250731585415</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707063092007568</v>
+        <v>4.707072093338335</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694411255786973</v>
+        <v>4.694420359596436</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678487261021663</v>
+        <v>4.678496443945066</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673496666753665</v>
+        <v>4.673505873450499</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686572783079335</v>
+        <v>4.686581990787879</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.70254706824634</v>
+        <v>4.70255815642261</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705703117392943</v>
+        <v>4.705710482157594</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694775887402308</v>
+        <v>4.694783395359496</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664813287966525</v>
+        <v>4.664821417879546</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649663160979965</v>
+        <v>4.649664472035953</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641417695705744</v>
+        <v>4.641420777018651</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636241737072735</v>
+        <v>4.636243639243669</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634028869759001</v>
+        <v>4.634033343756133</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637393968239524</v>
+        <v>4.637395092631743</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63441739952466</v>
+        <v>4.634414916871123</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627524326550192</v>
+        <v>4.627516841392991</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623778689886046</v>
+        <v>4.623770696030372</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599139192897209</v>
+        <v>4.599131321116753</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579438946040194</v>
+        <v>4.579422138157117</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560588250994405</v>
+        <v>4.560561113762132</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522479518074154</v>
+        <v>4.522439366192085</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519459038046687</v>
+        <v>4.519401951979581</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532230866615171</v>
+        <v>4.532167646462173</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551088231491788</v>
+        <v>4.551023775967634</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583549967555488</v>
+        <v>4.583477604212982</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.60208626833289</v>
+        <v>4.601993982859405</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674629763101535</v>
+        <v>4.674523895560846</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.710194960665286</v>
+        <v>4.710082684346405</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776944660348331</v>
+        <v>4.776838890306737</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812759469707357</v>
+        <v>4.812697408518222</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810521867505683</v>
+        <v>4.810461091171261</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819729552987704</v>
+        <v>4.819668810686816</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862320167533048</v>
+        <v>4.862314037784691</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855076862790468</v>
+        <v>4.855073311711221</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85311511203709</v>
+        <v>4.853143348938882</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.83024429794513</v>
+        <v>4.830264505592129</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838134023759035</v>
+        <v>4.838160669442901</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.89122364123207</v>
+        <v>4.891270891593461</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917736986070422</v>
+        <v>4.917765196911949</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926958129638141</v>
+        <v>4.926986749324343</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917065758435097</v>
+        <v>4.917093596717237</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897894412605767</v>
+        <v>4.897916774536728</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896255886508449</v>
+        <v>4.89629330482594</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896962293987137</v>
+        <v>4.897014783551464</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894366556645702</v>
+        <v>4.894436319612467</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878874355699407</v>
+        <v>4.87894616317078</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855482885463426</v>
+        <v>4.855543329240207</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829230219632698</v>
+        <v>4.829287932165462</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819968185336446</v>
+        <v>4.820023232611955</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789903293084866</v>
+        <v>4.789949309116114</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761960296099769</v>
+        <v>4.762006878606638</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.75105309702856</v>
+        <v>4.751100254435373</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755319145401227</v>
+        <v>4.755393501481963</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750104366305884</v>
+        <v>4.750150034385977</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750337396264429</v>
+        <v>4.750345055878194</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.75598382796027</v>
+        <v>4.755940250915504</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.76120354468628</v>
+        <v>4.761088647773846</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.769356946631756</v>
+        <v>4.769182498956591</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.775231050130876</v>
+        <v>4.775939462812498</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.773815533342352</v>
+        <v>4.774579100320691</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.773969965449256</v>
+        <v>4.774558079633414</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.771795006121531</v>
+        <v>4.77245068470631</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.77346104222134</v>
+        <v>4.774179459964322</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.779329503766722</v>
+        <v>4.780109267107374</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.80074397919816</v>
+        <v>4.801340809906507</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.814984921494941</v>
+        <v>4.815497316191761</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.826752858292267</v>
+        <v>4.82700875299923</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.829946316136876</v>
+        <v>4.830042387718479</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.848423254583714</v>
+        <v>4.847188981077837</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.850737672598219</v>
+        <v>4.848527300566899</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.846871488886876</v>
+        <v>4.843697033838591</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.815774623596267</v>
+        <v>4.813734259985734</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-17_00-28-44
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712822794924105</v>
+        <v>4.712822061936178</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711727505789939</v>
+        <v>4.711730918946983</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720255003612768</v>
+        <v>4.720259191983534</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707080916247112</v>
+        <v>4.70708956598591</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694429282960175</v>
+        <v>4.694438031189568</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678505444853908</v>
+        <v>4.678514269105784</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673514897707847</v>
+        <v>4.673523744894455</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686591016160743</v>
+        <v>4.68659986455999</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702569025869304</v>
+        <v>4.702579682993619</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705717701841291</v>
+        <v>4.70572478068848</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694790755342771</v>
+        <v>4.694797971683331</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664829387415424</v>
+        <v>4.664837201272646</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649665760622276</v>
+        <v>4.649667027297676</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64142380020382</v>
+        <v>4.641426766886952</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636245503872285</v>
+        <v>4.636247332059214</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634037729971316</v>
+        <v>4.63404203096178</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637396197182811</v>
+        <v>4.637397282405084</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634412484034884</v>
+        <v>4.634410099532982</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627509503195056</v>
+        <v>4.627502307672481</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623762859620419</v>
+        <v>4.623755176051031</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599123604840528</v>
+        <v>4.599116039507938</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579405669098357</v>
+        <v>4.579389528729251</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560534526759311</v>
+        <v>4.560508473440957</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522400024505943</v>
+        <v>4.522361468770622</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519346015014084</v>
+        <v>4.519291192848267</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532105693248929</v>
+        <v>4.532044969328701</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550960607534249</v>
+        <v>4.550898688091448</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583406678815278</v>
+        <v>4.583337149014279</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601903502460721</v>
+        <v>4.601814774759628</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674420101652844</v>
+        <v>4.674318321128056</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709972607892961</v>
+        <v>4.709864667366517</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776735158859405</v>
+        <v>4.776633407722212</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812636546070143</v>
+        <v>4.812576848018938</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810401481362963</v>
+        <v>4.810343004880487</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819609224907074</v>
+        <v>4.819550763014529</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862308016311268</v>
+        <v>4.862302100308092</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.85506981716348</v>
+        <v>4.855066377880479</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853171033871249</v>
+        <v>4.853198182852884</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830284307686486</v>
+        <v>4.830303716304182</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838186785880289</v>
+        <v>4.83821238866583</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891317213112</v>
+        <v>4.891362632895547</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917792835998214</v>
+        <v>4.917819920493252</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927014791709767</v>
+        <v>4.927042274037813</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917120889513086</v>
+        <v>4.917147652660228</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897938695501587</v>
+        <v>4.897960188374077</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896329999902931</v>
+        <v>4.896365992457541</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897066274439935</v>
+        <v>4.897116794804441</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894504745514153</v>
+        <v>4.894571872335349</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879016590466897</v>
+        <v>4.879085676933394</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855602599991688</v>
+        <v>4.855660731500767</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829344504193227</v>
+        <v>4.829399969162843</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820077187098883</v>
+        <v>4.820130080993676</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789994391358341</v>
+        <v>4.790038567873681</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762052536036956</v>
+        <v>4.762097295514415</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751146506072926</v>
+        <v>4.751191877555291</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755466523693963</v>
+        <v>4.755538247123325</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750194984646619</v>
+        <v>4.75023923287579</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.75035274333267</v>
+        <v>4.750360453046737</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755897685479015</v>
+        <v>4.755856098515022</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760976024259106</v>
+        <v>4.760865608780859</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.769011288798671</v>
+        <v>4.768843229218501</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.775736282841411</v>
+        <v>4.77553667739136</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.774721700285057</v>
+        <v>4.774764953077103</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.774516527101413</v>
+        <v>4.774372511339464</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.772304504347269</v>
+        <v>4.772059969725049</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.773731168819928</v>
+        <v>4.773213395540672</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.779585361688081</v>
+        <v>4.77897033169785</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.800359891021965</v>
+        <v>4.79929348259611</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.814058610410667</v>
+        <v>4.812543662903555</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.824887078419098</v>
+        <v>4.822718669952282</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.827039124415844</v>
+        <v>4.824039725386127</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.841836213289752</v>
+        <v>4.83668001746728</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.840725602633656</v>
+        <v>4.833412971764538</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.832392834050825</v>
+        <v>4.822234255989128</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.794972648053434</v>
+        <v>4.780198300153888</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.735272648053433</v>
+        <v>4.720498300153888</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-17_22-06-56
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.774764953077103</v>
+        <v>4.77399599973279</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.774372511339464</v>
+        <v>4.773472113402398</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.772059969725049</v>
+        <v>4.771099256626978</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.773213395540672</v>
+        <v>4.772238453090738</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.77897033169785</v>
+        <v>4.777841610314658</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.79929348259611</v>
+        <v>4.798000762173006</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.812543662903555</v>
+        <v>4.811044428605653</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.822718669952282</v>
+        <v>4.821019494597314</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.824039725386127</v>
+        <v>4.82202756011475</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.83668001746728</v>
+        <v>4.834165193883592</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.833412971764538</v>
+        <v>4.830186652045075</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.822234255989128</v>
+        <v>4.817735219854609</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.780198300153888</v>
+        <v>4.771868209624516</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.720498300153888</v>
+        <v>4.698765709624516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-18_22-08-58
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712822061936178</v>
+        <v>4.712821343179671</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711730918946983</v>
+        <v>4.711734265522548</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720259191983534</v>
+        <v>4.720263299130833</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70708956598591</v>
+        <v>4.707098047602642</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694438031189568</v>
+        <v>4.694446609389599</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678514269105784</v>
+        <v>4.67852292185009</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673523744894455</v>
+        <v>4.673532420170496</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68659986455999</v>
+        <v>4.686608541139512</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702579682993619</v>
+        <v>4.70259013395499</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70572478068848</v>
+        <v>4.705731722779671</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694797971683331</v>
+        <v>4.694805048545001</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664837201272646</v>
+        <v>4.664844863967964</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649667027297676</v>
+        <v>4.649668272603133</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641426766886952</v>
+        <v>4.641429678633832</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636247332059214</v>
+        <v>4.636249124862475</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.63404203096178</v>
+        <v>4.634046249186428</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637397282405084</v>
+        <v>4.637398348793782</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634410099532982</v>
+        <v>4.63440776194067</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627502307672481</v>
+        <v>4.627495250706187</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623755176051031</v>
+        <v>4.623747640894878</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599116039507938</v>
+        <v>4.599108620734915</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579389528729251</v>
+        <v>4.579373707315007</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560508473440957</v>
+        <v>4.560482937918027</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522361468770622</v>
+        <v>4.522323675697628</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519291192848267</v>
+        <v>4.519237452530209</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532044969328701</v>
+        <v>4.531985438529427</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550898688091448</v>
+        <v>4.550837981025458</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583337149014279</v>
+        <v>4.583268974105188</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601814774759628</v>
+        <v>4.601727749383237</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674318321128056</v>
+        <v>4.674218496045475</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709864667366517</v>
+        <v>4.709758801279291</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776633407722212</v>
+        <v>4.77653358080839</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812576848018938</v>
+        <v>4.812518281317842</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810343004880487</v>
+        <v>4.810285629769036</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819550763014529</v>
+        <v>4.819493393588299</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862302100308092</v>
+        <v>4.862296287064867</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855066377880479</v>
+        <v>4.855062992629648</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853198182852884</v>
+        <v>4.853224811288928</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830303716304182</v>
+        <v>4.830322743046892</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83821238866583</v>
+        <v>4.838237492788135</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891362632895547</v>
+        <v>4.891407177007828</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917819920493252</v>
+        <v>4.917846466882511</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927042274037813</v>
+        <v>4.927069212873785</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917147652660228</v>
+        <v>4.917173901390561</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897960188374077</v>
+        <v>4.897981265533254</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896365992457541</v>
+        <v>4.896401302425969</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897116794804441</v>
+        <v>4.897166371751756</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894571872335349</v>
+        <v>4.894637736638761</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879085676933394</v>
+        <v>4.879153460436984</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855660731500767</v>
+        <v>4.855717756266777</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829399969162843</v>
+        <v>4.829454359227157</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820130080993676</v>
+        <v>4.82018194524125</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790038567873681</v>
+        <v>4.790081865613848</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762097295514415</v>
+        <v>4.762141183118681</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751191877555291</v>
+        <v>4.751236393548732</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755538247123325</v>
+        <v>4.755608705655844</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.75023923287579</v>
+        <v>4.750282794446937</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750360453046737</v>
+        <v>4.750368179819505</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755856098515022</v>
+        <v>4.755815458267891</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760865608780859</v>
+        <v>4.760757338406883</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.768843229218501</v>
+        <v>4.768678236271506</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.77553667739136</v>
+        <v>4.775340556496596</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.77399599973279</v>
+        <v>4.773560492529362</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.773472113402398</v>
+        <v>4.772779355044982</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.771099256626978</v>
+        <v>4.770292180341156</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.772238453090738</v>
+        <v>4.771193829142514</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.777841610314658</v>
+        <v>4.776601528284417</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.798000762173006</v>
+        <v>4.796241028175613</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.811044428605653</v>
+        <v>4.808751948069821</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.821019494597314</v>
+        <v>4.818012721849925</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.82202756011475</v>
+        <v>4.818106892957955</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.834165193883592</v>
+        <v>4.828078170196537</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.830186652045075</v>
+        <v>4.821949104267077</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.817735219854609</v>
+        <v>4.806776502953907</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.771868209624516</v>
+        <v>4.757201465603789</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.698765709624516</v>
+        <v>4.631126911225324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-19_12-33-32
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712821343179671</v>
+        <v>4.712820638244114</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711734265522548</v>
+        <v>4.711737547445895</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720263299130833</v>
+        <v>4.720267327394351</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707098047602642</v>
+        <v>4.707106365950946</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694446609389599</v>
+        <v>4.694455022468786</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.67852292185009</v>
+        <v>4.67853140803805</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673532420170496</v>
+        <v>4.6735409284976</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686608541139512</v>
+        <v>4.686617050855028</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.70259013395499</v>
+        <v>4.702600384676949</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705731722779671</v>
+        <v>4.705738532039268</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694805048545001</v>
+        <v>4.694811989932239</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664844863967964</v>
+        <v>4.664852379845103</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649668272603133</v>
+        <v>4.64966949706254</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641429678633832</v>
+        <v>4.64143253695306</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636249124862475</v>
+        <v>4.636250883299522</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634046249186428</v>
+        <v>4.634050387010514</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637398348793782</v>
+        <v>4.637399396827679</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63440776194067</v>
+        <v>4.634405469888605</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627495250706187</v>
+        <v>4.627488328334071</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623747640894878</v>
+        <v>4.623740249893954</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599108620734915</v>
+        <v>4.599101344305458</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579373707315007</v>
+        <v>4.579358195501205</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560482937918027</v>
+        <v>4.560457904925265</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522323675697628</v>
+        <v>4.522286622908412</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519237452530209</v>
+        <v>4.519184762392313</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531985438529427</v>
+        <v>4.531927066082307</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550837981025458</v>
+        <v>4.55077845113726</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583268974105188</v>
+        <v>4.583202114947723</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601727749383237</v>
+        <v>4.601642377868139</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674218496045475</v>
+        <v>4.674120570663199</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709758801279291</v>
+        <v>4.709654950478018</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.77653358080839</v>
+        <v>4.776435624126115</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812518281317842</v>
+        <v>4.812460814156937</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810285629769036</v>
+        <v>4.810229325261584</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819493393588299</v>
+        <v>4.819437086364895</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862296287064867</v>
+        <v>4.862290573961843</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855062992629648</v>
+        <v>4.855059660211683</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853224811288928</v>
+        <v>4.85325093400006</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830322743046892</v>
+        <v>4.830341399065039</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838237492788135</v>
+        <v>4.838262112658921</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891407177007828</v>
+        <v>4.891450870518203</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917846466882511</v>
+        <v>4.917872491005975</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927069212873785</v>
+        <v>4.927095624137809</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917173901390561</v>
+        <v>4.917199650358907</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897981265533254</v>
+        <v>4.898001938886938</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896401302425969</v>
+        <v>4.896435948998937</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897166371751756</v>
+        <v>4.897215031391436</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894637736638761</v>
+        <v>4.894702373630968</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879153460436984</v>
+        <v>4.879219977434183</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855717756266777</v>
+        <v>4.855773705565825</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829454359227157</v>
+        <v>4.82950770530692</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.82018194524125</v>
+        <v>4.82023280959517</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790081865613848</v>
+        <v>4.790124310474388</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762141183118681</v>
+        <v>4.762184223934845</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751236393548732</v>
+        <v>4.751280077814716</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755608705655844</v>
+        <v>4.755677932026931</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750282794446937</v>
+        <v>4.750325684329837</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750368179819505</v>
+        <v>4.750375918805244</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755815458267891</v>
+        <v>4.755775734293078</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760757338406883</v>
+        <v>4.760651152524556</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.768678236271506</v>
+        <v>4.768516228884561</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.775340556496596</v>
+        <v>4.775147833046168</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.773560492529362</v>
+        <v>4.773113760866418</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.772779355044982</v>
+        <v>4.772036326781618</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.770292180341156</v>
+        <v>4.769423743678955</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.771193829142514</v>
+        <v>4.770021433879817</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.776601528284417</v>
+        <v>4.775225481149564</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.796241028175613</v>
+        <v>4.794272760337089</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.808751948069821</v>
+        <v>4.806161700346776</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.818012721849925</v>
+        <v>4.814644404088465</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.818106892957955</v>
+        <v>4.813766750700679</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.828078170196537</v>
+        <v>4.821633277821597</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.821949104267077</v>
+        <v>4.813701416681653</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.806776502953907</v>
+        <v>4.796312105974209</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.757201465603789</v>
+        <v>4.744437512279664</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.631126911225324</v>
+        <v>4.628683330381645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-21_20-34-41
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712820638244114</v>
+        <v>4.712819946734673</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711737547445895</v>
+        <v>4.711740766572464</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720267327394351</v>
+        <v>4.72027127902478</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707106365950946</v>
+        <v>4.70711452569944</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694455022468786</v>
+        <v>4.694463275148543</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.67853140803805</v>
+        <v>4.678539732432151</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.6735409284976</v>
+        <v>4.67354927464831</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686617050855028</v>
+        <v>4.686625398473527</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702600384676949</v>
+        <v>4.702610440858309</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705738532039268</v>
+        <v>4.70574521224297</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694811989932239</v>
+        <v>4.694818799697693</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664852379845103</v>
+        <v>4.66485975308297</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64966949706254</v>
+        <v>4.64967070118334</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64143253695306</v>
+        <v>4.641435343298628</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636250883299522</v>
+        <v>4.636252608349171</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634050387010514</v>
+        <v>4.634054446710055</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637399396827679</v>
+        <v>4.637400426969767</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634405469888605</v>
+        <v>4.634403222060172</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627488328334071</v>
+        <v>4.627481536743604</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623740249893954</v>
+        <v>4.623732998951557</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599101344305458</v>
+        <v>4.599094206163659</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579358195501205</v>
+        <v>4.579342984295403</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560457904925265</v>
+        <v>4.560433359790931</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522286622908412</v>
+        <v>4.522250288890417</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519184762392313</v>
+        <v>4.519133091989417</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531927066082307</v>
+        <v>4.531869818554519</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.55077845113726</v>
+        <v>4.550720064575027</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583202114947723</v>
+        <v>4.583136533891815</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601642377868139</v>
+        <v>4.601558613570901</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.674120570663199</v>
+        <v>4.674024491335219</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709654950478018</v>
+        <v>4.709553058034349</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776435624126115</v>
+        <v>4.776339485681754</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812460814156937</v>
+        <v>4.812404415905906</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810229325261584</v>
+        <v>4.810174061724307</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819437086364895</v>
+        <v>4.819381812185545</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862290573961843</v>
+        <v>4.862284958466151</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855059660211683</v>
+        <v>4.85505637945961</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85325093400006</v>
+        <v>4.853276565249925</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830341399065039</v>
+        <v>4.830359695079491</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838262112658921</v>
+        <v>4.838286262140475</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891450870518203</v>
+        <v>4.891493737548624</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917872491005975</v>
+        <v>4.917898008089381</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927095624137809</v>
+        <v>4.927121523135863</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917199650358907</v>
+        <v>4.917224913670019</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898001938886938</v>
+        <v>4.898022219893873</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896435948998937</v>
+        <v>4.896469950656133</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897215031391436</v>
+        <v>4.897262798881126</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894702373630968</v>
+        <v>4.894765817224568</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879219977434183</v>
+        <v>4.879285263036234</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855773705565825</v>
+        <v>4.85582860950773</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.82950770530692</v>
+        <v>4.829560037149205</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.82023280959517</v>
+        <v>4.820282702674391</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790124310474388</v>
+        <v>4.790165927345795</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762184223934845</v>
+        <v>4.762226442100145</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751280077814716</v>
+        <v>4.751322953250623</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755677932026931</v>
+        <v>4.755745957869102</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750325684329837</v>
+        <v>4.750367917101308</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750375918805244</v>
+        <v>4.75038366549008</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755775734293078</v>
+        <v>4.75573689739206</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760651152524556</v>
+        <v>4.760546992737225</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.768516228884561</v>
+        <v>4.768357128738307</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.775147833046168</v>
+        <v>4.77495842267859</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.773113760866418</v>
+        <v>4.772691485654414</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.772036326781618</v>
+        <v>4.771329467447343</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.769423743678955</v>
+        <v>4.768597646953393</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.770021433879817</v>
+        <v>4.768881829974932</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.775225481149564</v>
+        <v>4.77391268212121</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.794272760337089</v>
+        <v>4.792395605941822</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.806161700346776</v>
+        <v>4.803699428456766</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.814644404088465</v>
+        <v>4.811454843198721</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.813766750700679</v>
+        <v>4.809689703857327</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.821633277821597</v>
+        <v>4.81564650624446</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.813701416681653</v>
+        <v>4.806169685345673</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.796312105974209</v>
+        <v>4.787034482197933</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.744437512279664</v>
+        <v>4.734002231109966</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.628683330381645</v>
+        <v>4.627197389614509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-23_20-36-52
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712819268271407</v>
+        <v>4.712818602488578</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711743924687376</v>
+        <v>4.71174702350873</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720275156188006</v>
+        <v>4.720278960969068</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707122531340452</v>
+        <v>4.707130387198259</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694471371972002</v>
+        <v>4.694479317312356</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678547899615051</v>
+        <v>4.678555913997983</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673557463215005</v>
+        <v>4.673565498618316</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686633588582154</v>
+        <v>4.68664162559662</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702620307983715</v>
+        <v>4.702629991333617</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705751767024746</v>
+        <v>4.705758199883419</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694825481549318</v>
+        <v>4.694832039057115</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664866987703389</v>
+        <v>4.664874087578422</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649671885457132</v>
+        <v>4.649673050360263</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641438099072367</v>
+        <v>4.641440805626253</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636254300953411</v>
+        <v>4.636255962019124</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634058430476001</v>
+        <v>4.634062340418169</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637401439667873</v>
+        <v>4.637402435355276</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634401017188971</v>
+        <v>4.634398854056458</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627474872264831</v>
+        <v>4.627468331363794</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623725884124729</v>
+        <v>4.623718901617108</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599087202406187</v>
+        <v>4.599080329275173</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579328065049807</v>
+        <v>4.579313429444933</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560409288408259</v>
+        <v>4.560385677208549</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522214652955633</v>
+        <v>4.522179695201507</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519082412040445</v>
+        <v>4.519032694373363</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531813663785742</v>
+        <v>4.531758570828275</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550662788770381</v>
+        <v>4.550606592378253</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583072194707492</v>
+        <v>4.583009062518678</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601476411583527</v>
+        <v>4.601395728653599</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.67393020641396</v>
+        <v>4.673837666158208</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.70945306914135</v>
+        <v>4.709354931015733</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776245115388401</v>
+        <v>4.776152464979417</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812349057059942</v>
+        <v>4.812294709188609</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.81011981060499</v>
+        <v>4.810066544384219</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819327542946397</v>
+        <v>4.819274251551343</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862279438128301</v>
+        <v>4.862274010578842</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855053149237875</v>
+        <v>4.855049968441459</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853301718771062</v>
+        <v>4.853326407789369</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830377641402041</v>
+        <v>4.830395247954713</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838309954571551</v>
+        <v>4.838333202791841</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891535801317938</v>
+        <v>4.891577084183742</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917923032773646</v>
+        <v>4.917947579142615</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927146924589033</v>
+        <v>4.927171842661123</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.91724970490408</v>
+        <v>4.917274037140812</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898042119584618</v>
+        <v>4.898061648581315</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896503325198761</v>
+        <v>4.896536089780323</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897309698469414</v>
+        <v>4.897355753536404</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894828100096943</v>
+        <v>4.894889253745867</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879349351070491</v>
+        <v>4.879412274138488</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855882497089841</v>
+        <v>4.855935396247892</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829611383382521</v>
+        <v>4.829661771568849</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820331652016795</v>
+        <v>4.820379684129719</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790206740161679</v>
+        <v>4.79024677194421</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762267860848055</v>
+        <v>4.762308502549976</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751365041928306</v>
+        <v>4.751406365130621</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755812813757204</v>
+        <v>4.755878529251479</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750409506955799</v>
+        <v>4.750450467715767</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750391415670313</v>
+        <v>4.750399165432231</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755698919551023</v>
+        <v>4.755661773883039</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760444802765935</v>
+        <v>4.760344528356241</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.768200860154975</v>
+        <v>4.768047349991429</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.774772243680694</v>
+        <v>4.774589216890515</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.772504770583834</v>
+        <v>4.772320935018032</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.770886581242098</v>
+        <v>4.770529183018852</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.768002755801426</v>
+        <v>4.767514405775209</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.768220029257687</v>
+        <v>4.767687341146736</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.772651556335423</v>
+        <v>4.771544891018843</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.790612431762356</v>
+        <v>4.78900114071401</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.801409938416409</v>
+        <v>4.799316596393632</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.808579379069228</v>
+        <v>4.805930236665679</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.806147951829299</v>
+        <v>4.802883591573421</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.810850646475787</v>
+        <v>4.806437456895225</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.799973783169079</v>
+        <v>4.794294214737096</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.779609026932976</v>
+        <v>4.7729178727826</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.726447349194188</v>
+        <v>4.71994749574417</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.628209549198851</v>
+        <v>4.628590760926228</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.609552104956753</v>
+        <v>4.608059348618127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-24_20-36-02
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712818602488578</v>
+        <v>4.712817949033995</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.71174702350873</v>
+        <v>4.711750064690726</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720278960969068</v>
+        <v>4.7202826953759</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707130387198259</v>
+        <v>4.707138097436881</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694479317312356</v>
+        <v>4.694487115380727</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678555913997983</v>
+        <v>4.678563779828701</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673565498618316</v>
+        <v>4.673573385115089</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68664162559662</v>
+        <v>4.68664951376913</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702629991333617</v>
+        <v>4.702639495993671</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705758199883419</v>
+        <v>4.705764514188891</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694832039057115</v>
+        <v>4.694838475659474</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664874087578422</v>
+        <v>4.66488105643726</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649673050360263</v>
+        <v>4.649674196354388</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641440805626253</v>
+        <v>4.641443464264606</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636255962019124</v>
+        <v>4.636257592419707</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634062340418169</v>
+        <v>4.634066178568966</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637402435355276</v>
+        <v>4.637403414451267</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634398854056458</v>
+        <v>4.6343967314897</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627468331363794</v>
+        <v>4.627461910636266</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623718901617108</v>
+        <v>4.62371204777218</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599080329275173</v>
+        <v>4.599073583151505</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579313429444933</v>
+        <v>4.579299069474187</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560385677208549</v>
+        <v>4.560362513135789</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522179695201507</v>
+        <v>4.522145396474071</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519032694373363</v>
+        <v>4.518983911873225</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531758570828275</v>
+        <v>4.531704509890488</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550606592378253</v>
+        <v>4.550551445220053</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.583009062518678</v>
+        <v>4.582947103740654</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601395728653599</v>
+        <v>4.601316523108768</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673837666158208</v>
+        <v>4.67374682264606</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709354931015733</v>
+        <v>4.709258592805416</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776152464979417</v>
+        <v>4.776061487926592</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812294709188609</v>
+        <v>4.812241344887452</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810066544384219</v>
+        <v>4.810014236529192</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819274251551343</v>
+        <v>4.819221911867393</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862274010578842</v>
+        <v>4.862268673525193</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855049968441459</v>
+        <v>4.855046835994989</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853326407789369</v>
+        <v>4.853350645047248</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830395247954713</v>
+        <v>4.830412524287988</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838333202791841</v>
+        <v>4.838356019165063</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891577084183742</v>
+        <v>4.891617607681935</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917947579142615</v>
+        <v>4.917971660749255</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927171842661123</v>
+        <v>4.92719629098471</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917274037140812</v>
+        <v>4.917297922982263</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898061648581315</v>
+        <v>4.898080817116355</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896536089780323</v>
+        <v>4.896568260935739</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897355753536404</v>
+        <v>4.897400986632151</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894889253745867</v>
+        <v>4.894949308542131</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879412274138488</v>
+        <v>4.879474063670861</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855935396247892</v>
+        <v>4.855987333904096</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829661771568849</v>
+        <v>4.82971122825282</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820379684129719</v>
+        <v>4.820426824537684</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.79024677194421</v>
+        <v>4.790286044846999</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762308502549976</v>
+        <v>4.762348388754641</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751406365130621</v>
+        <v>4.751446943386055</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755878529251479</v>
+        <v>4.755943132938585</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750450467715767</v>
+        <v>4.750490812841899</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750399165432231</v>
+        <v>4.750406911133323</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755661773883039</v>
+        <v>4.755625434573528</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760344528356241</v>
+        <v>4.760246117189794</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.768047349991429</v>
+        <v>4.767896527537168</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.774589216890515</v>
+        <v>4.774409265604064</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.772320935018032</v>
+        <v>4.772139917237881</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.770529183018852</v>
+        <v>4.76908000816995</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.767514405775209</v>
+        <v>4.765758163347808</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.767687341146736</v>
+        <v>4.765708199408044</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.771544891018843</v>
+        <v>4.769172878917241</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.78900114071401</v>
+        <v>4.785882860656235</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.799316596393632</v>
+        <v>4.795468013974928</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.805930236665679</v>
+        <v>4.801286302280978</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.802883591573421</v>
+        <v>4.797274680754014</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.806437456895225</v>
+        <v>4.799259595473277</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.794294214737096</v>
+        <v>4.785167946608281</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.7729178727826</v>
+        <v>4.761850651780835</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.71994749574417</v>
+        <v>4.706898901210443</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.628590760926228</v>
+        <v>4.615798017634265</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.608059348618127</v>
+        <v>4.572483065817394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add forecast evidence lifecycle dashboard
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712817949033995</v>
+        <v>4.712817307568386</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711750064690726</v>
+        <v>4.711753049826596</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.7202826953759</v>
+        <v>4.720286361342851</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707138097436881</v>
+        <v>4.707145666067427</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694487115380727</v>
+        <v>4.694494770233604</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678563779828701</v>
+        <v>4.678571501198977</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673573385115089</v>
+        <v>4.673581126805892</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68664951376913</v>
+        <v>4.686657257195884</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702639495993671</v>
+        <v>4.702648826863644</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705764514188891</v>
+        <v>4.705770713188028</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694838475659474</v>
+        <v>4.694844794669192</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.66488105643726</v>
+        <v>4.664887897872768</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649674196354388</v>
+        <v>4.649675323887008</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641443464264606</v>
+        <v>4.641446076246158</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636257592419707</v>
+        <v>4.636259192996596</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634066178568966</v>
+        <v>4.634069946886896</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637403414451267</v>
+        <v>4.637404377361699</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.6343967314897</v>
+        <v>4.63439464835926</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627461910636266</v>
+        <v>4.627455606801873</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62371204777218</v>
+        <v>4.623705319066906</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599073583151505</v>
+        <v>4.599066960548487</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579299069474187</v>
+        <v>4.579284977429294</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560362513135789</v>
+        <v>4.560339783622692</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522145396474071</v>
+        <v>4.522111738333104</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518983911873225</v>
+        <v>4.518936038433111</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531704509890488</v>
+        <v>4.531651452283416</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550551445220053</v>
+        <v>4.550497318230012</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582947103740654</v>
+        <v>4.582886286020946</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601316523108768</v>
+        <v>4.601238754785349</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.67374682264606</v>
+        <v>4.67365762969261</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709258592805416</v>
+        <v>4.709164005502117</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.776061487926592</v>
+        <v>4.775972139362694</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812241344887452</v>
+        <v>4.812188937732199</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810014236529192</v>
+        <v>4.80996286144998</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819221911867393</v>
+        <v>4.81917049868234</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862268673525193</v>
+        <v>4.862263424748596</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855046835994989</v>
+        <v>4.855043750851891</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853350645047248</v>
+        <v>4.853374442825494</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830412524287988</v>
+        <v>4.830429479598028</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838356019165063</v>
+        <v>4.838378415600801</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891617607681935</v>
+        <v>4.891657392564094</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917971660749255</v>
+        <v>4.917995290640382</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.92719629098471</v>
+        <v>4.927220282685758</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917297922982263</v>
+        <v>4.917321374574364</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898080817116355</v>
+        <v>4.898099635050042</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896568260935739</v>
+        <v>4.896599854608928</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897400986632151</v>
+        <v>4.897445419513056</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.894949308542131</v>
+        <v>4.895008293779392</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879474063670861</v>
+        <v>4.879534749979372</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855987333904096</v>
+        <v>4.856038336012653</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.82971122825282</v>
+        <v>4.829759779008176</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820426824537684</v>
+        <v>4.820473097827497</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790286044846999</v>
+        <v>4.790324580195586</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762348388754641</v>
+        <v>4.762387540225383</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751446943386055</v>
+        <v>4.751486796501561</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.755943132938585</v>
+        <v>4.756006652470683</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750490812841899</v>
+        <v>4.750530555443125</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750406911133323</v>
+        <v>4.750414649384773</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755625434573528</v>
+        <v>4.755589876828764</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760246117189794</v>
+        <v>4.760149518800404</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.767896527537168</v>
+        <v>4.767748324417025</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.774409265604064</v>
+        <v>4.774232315485795</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.772139917237881</v>
+        <v>4.77196165709638</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.76908000816995</v>
+        <v>4.767696039007633</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.765758163347808</v>
+        <v>4.764187676730078</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.765708199408044</v>
+        <v>4.763907869745815</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.769172878917241</v>
+        <v>4.766976832075328</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.785882860656235</v>
+        <v>4.783066046645596</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.795468013974928</v>
+        <v>4.792018037207778</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.801286302280978</v>
+        <v>4.79712750031236</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.797274680754014</v>
+        <v>4.792259778018465</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.799259595473277</v>
+        <v>4.792848088694397</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.785167946608281</v>
+        <v>4.777097083658976</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.761850651780835</v>
+        <v>4.752276125272326</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.706898901210443</v>
+        <v>4.696245896205808</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.615798017634265</v>
+        <v>4.606812641185805</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.572483065817394</v>
+        <v>4.556525494599769</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-25_20-37-23
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.767696039007633</v>
+        <v>4.767335055906479</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.764187676730078</v>
+        <v>4.763774736928711</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.763907869745815</v>
+        <v>4.763457401996668</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.766976832075328</v>
+        <v>4.766472384924684</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.783066046645596</v>
+        <v>4.78253031464685</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.792018037207778</v>
+        <v>4.791419772661629</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.79712750031236</v>
+        <v>4.796462389380321</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.792259778018465</v>
+        <v>4.791486160236009</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.792848088694397</v>
+        <v>4.791931418845788</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.777097083658976</v>
+        <v>4.775950092407074</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.752276125272326</v>
+        <v>4.750826421458777</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.696245896205808</v>
+        <v>4.694162392481778</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.606812641185805</v>
+        <v>4.603374340958304</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.556525494599769</v>
+        <v>4.548758038122479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-26_09-38-15
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712817307568386</v>
+        <v>4.712816677764813</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711753049826596</v>
+        <v>4.711755980451395</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720286361342851</v>
+        <v>4.720289960734035</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707145666067427</v>
+        <v>4.707153096955049</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694494770233604</v>
+        <v>4.694502285779874</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678571501198977</v>
+        <v>4.678579082051701</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673581126805892</v>
+        <v>4.673588727642117</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686657257195884</v>
+        <v>4.686664859824165</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702648826863644</v>
+        <v>4.702657988665831</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705770713188028</v>
+        <v>4.705776800010221</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694844794669192</v>
+        <v>4.694850999279153</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664887897872768</v>
+        <v>4.664894615347644</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649675323887008</v>
+        <v>4.649676433391994</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641446076246158</v>
+        <v>4.641448642786033</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636259192996596</v>
+        <v>4.636260764560724</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634069946886896</v>
+        <v>4.634073647259902</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637404377361699</v>
+        <v>4.637405324479514</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63439464835926</v>
+        <v>4.634392603577212</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627455606801873</v>
+        <v>4.627449416698511</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623705319066906</v>
+        <v>4.623698712105675</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599066960548487</v>
+        <v>4.599060458105832</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579284977429294</v>
+        <v>4.579271145886548</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560339783622692</v>
+        <v>4.560317476568055</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522111738333104</v>
+        <v>4.52207870301923</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518936038433111</v>
+        <v>4.518889048907768</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531651452283416</v>
+        <v>4.531599370370278</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550497318230012</v>
+        <v>4.550444183404426</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582886286020946</v>
+        <v>4.582826578183428</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601238754785349</v>
+        <v>4.601162384960733</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.67365762969261</v>
+        <v>4.673570042772052</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.709164005502117</v>
+        <v>4.70907112185864</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775972139362694</v>
+        <v>4.775884376008118</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812188937732199</v>
+        <v>4.812137462235389</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.80996286144998</v>
+        <v>4.809912394458091</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.81917049868234</v>
+        <v>4.81911998766468</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862263424748596</v>
+        <v>4.86225826210123</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855043750851891</v>
+        <v>4.855040711993553</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853374442825494</v>
+        <v>4.853397812963987</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830429479598028</v>
+        <v>4.830446122742938</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838378415600801</v>
+        <v>4.838400403575134</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891657392564094</v>
+        <v>4.891696458832852</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917995290640382</v>
+        <v>4.918018481380027</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927220282685758</v>
+        <v>4.927243830406889</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917321374574364</v>
+        <v>4.917344403627334</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898099635050042</v>
+        <v>4.898118111887308</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896599854608928</v>
+        <v>4.896630886178917</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897445419513056</v>
+        <v>4.897489073176394</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895008293779392</v>
+        <v>4.895066237721409</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879534749979372</v>
+        <v>4.879594362306189</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856038336012653</v>
+        <v>4.856088427602831</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829759779008176</v>
+        <v>4.829807448481734</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820473097827497</v>
+        <v>4.820518527690888</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790324580195586</v>
+        <v>4.790362398525678</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762387540225383</v>
+        <v>4.762425976975427</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751486796501561</v>
+        <v>4.751525943593718</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756006652470683</v>
+        <v>4.756069114602697</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750530555443125</v>
+        <v>4.750569708286424</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750414649384773</v>
+        <v>4.750422377035134</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755589876828764</v>
+        <v>4.755555076827278</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760149518800404</v>
+        <v>4.760054684494373</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.767748324417025</v>
+        <v>4.767602674498344</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.774232315485795</v>
+        <v>4.774058294482692</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.77196165709638</v>
+        <v>4.771786095978607</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.767335055906479</v>
+        <v>4.765666579272082</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.763774736928711</v>
+        <v>4.76187841894254</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.763457401996668</v>
+        <v>4.761305354994633</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.766472384924684</v>
+        <v>4.76389096211962</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.78253031464685</v>
+        <v>4.779331302407662</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.791419772661629</v>
+        <v>4.787568624849621</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.796462389380321</v>
+        <v>4.791885249516502</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.791486160236009</v>
+        <v>4.786023404430199</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.791931418845788</v>
+        <v>4.785067382525204</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.775950092407074</v>
+        <v>4.767414644809636</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.750826421458777</v>
+        <v>4.740804520453976</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.694162392481778</v>
+        <v>4.683051925319735</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.603374340958304</v>
+        <v>4.593454552431115</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.548758038122479</v>
+        <v>4.534535381480097</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-28_20-38-16
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712816677764813</v>
+        <v>4.712816059308125</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711755980451395</v>
+        <v>4.711758858044636</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720289960734035</v>
+        <v>4.720293495346483</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707153096955049</v>
+        <v>4.707160393825526</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694502285779874</v>
+        <v>4.694509665787476</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678579082051701</v>
+        <v>4.678586526187582</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673588727642117</v>
+        <v>4.67359619143271</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686664859824165</v>
+        <v>4.686672325459038</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702657988665831</v>
+        <v>4.702666985953012</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705776800010221</v>
+        <v>4.705782777672652</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694850999279153</v>
+        <v>4.694857092567699</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664894615347644</v>
+        <v>4.66490121220027</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649676433391994</v>
+        <v>4.649677525290071</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641448642786033</v>
+        <v>4.641451165057606</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636260764560724</v>
+        <v>4.636262307893886</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634073647259902</v>
+        <v>4.634077281508503</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637405324479514</v>
+        <v>4.637406256185238</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634392603577212</v>
+        <v>4.634390596095246</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627449416698511</v>
+        <v>4.627443337277058</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623698712105675</v>
+        <v>4.62369222361461</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599060458105832</v>
+        <v>4.599054072584001</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579271145886548</v>
+        <v>4.579257567693807</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560317476568055</v>
+        <v>4.560295580315382</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.52207870301923</v>
+        <v>4.522046273422818</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518889048907768</v>
+        <v>4.518842919069789</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531599370370278</v>
+        <v>4.531548237518736</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550444183404426</v>
+        <v>4.55039201375366</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582826578183428</v>
+        <v>4.582767950175429</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601162384960733</v>
+        <v>4.60108737628941</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673570042772052</v>
+        <v>4.673484018943933</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.70907112185864</v>
+        <v>4.70897989631057</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775884376008118</v>
+        <v>4.775798156101363</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812137462235389</v>
+        <v>4.812086893805286</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809912394458091</v>
+        <v>4.809862811727189</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.81911998766468</v>
+        <v>4.819070355325569</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86225826210123</v>
+        <v>4.862253183503444</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855040711993553</v>
+        <v>4.855037718428507</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853397812963987</v>
+        <v>4.853420766881301</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830446122742938</v>
+        <v>4.830462462258145</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838400403575134</v>
+        <v>4.838421994150176</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891696458832852</v>
+        <v>4.891734825775365</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918018481380027</v>
+        <v>4.918041245071505</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927243830406889</v>
+        <v>4.927266946329362</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917344403627334</v>
+        <v>4.917367021435004</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898118111887308</v>
+        <v>4.898136256793526</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896630886178917</v>
+        <v>4.896661370484582</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897489073176394</v>
+        <v>4.897531967893042</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895066237721409</v>
+        <v>4.8951231676468</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879594362306189</v>
+        <v>4.879652928870575</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856088427602831</v>
+        <v>4.856137632819761</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829807448481734</v>
+        <v>4.829854260434959</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820518527690888</v>
+        <v>4.820563136964852</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790362398525678</v>
+        <v>4.790399519619315</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762425976975427</v>
+        <v>4.76246371830128</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751525943593718</v>
+        <v>4.751564403118288</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756069114602697</v>
+        <v>4.756130545227847</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750569708286424</v>
+        <v>4.750608283806415</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750422377035134</v>
+        <v>4.750430091155124</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755555076827278</v>
+        <v>4.755521011673922</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.760054684494373</v>
+        <v>4.759961567274797</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.767602674498344</v>
+        <v>4.767459513802372</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.774058294482692</v>
+        <v>4.773887132741752</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.771786095978607</v>
+        <v>4.771613176762193</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.765666579272082</v>
+        <v>4.764415028856755</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.76187841894254</v>
+        <v>4.760473105232219</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.761305354994633</v>
+        <v>4.759732586237501</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.76389096211962</v>
+        <v>4.761951807267181</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.779331302407662</v>
+        <v>4.776851284838035</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.787568624849621</v>
+        <v>4.784539759745135</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.791885249516502</v>
+        <v>4.788245895803191</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.786023404430199</v>
+        <v>4.781684907764487</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.785067382525204</v>
+        <v>4.779605826461957</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.767414644809636</v>
+        <v>4.760739620398042</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.740804520453976</v>
+        <v>4.73323986677563</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.683051925319735</v>
+        <v>4.675515934664416</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.593454552431115</v>
+        <v>4.588841619962075</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.534535381480097</v>
+        <v>4.531562681903836</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-01_00-09-07
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712815451894418</v>
+        <v>4.712814855230546</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711761684032766</v>
+        <v>4.711764459791539</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720296966913136</v>
+        <v>4.720300377105684</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707167560271485</v>
+        <v>4.707174599758295</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694516913889694</v>
+        <v>4.694524033591122</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678593837271508</v>
+        <v>4.678601018838553</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673603521850532</v>
+        <v>4.673610722438372</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686679657769708</v>
+        <v>4.68668686029552</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702675823115986</v>
+        <v>4.702684504390717</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705788649085278</v>
+        <v>4.705794417055547</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694863077503729</v>
+        <v>4.694868956951511</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664907691650231</v>
+        <v>4.664914056803559</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649678599989306</v>
+        <v>4.649679657885559</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641453644194279</v>
+        <v>4.641456081291172</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636263823750038</v>
+        <v>4.636265312856521</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634080851388779</v>
+        <v>4.634084358595198</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637407172847457</v>
+        <v>4.637408074823274</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634388624902878</v>
+        <v>4.634386689025769</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627437365596385</v>
+        <v>4.627431498818609</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623685850436147</v>
+        <v>4.623679589523932</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599047800858815</v>
+        <v>4.599041639916377</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.5792442359582</v>
+        <v>4.579231144034479</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560274083632661</v>
+        <v>4.560252975693226</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522014433054569</v>
+        <v>4.521983166017675</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518797625568149</v>
+        <v>4.518753145888986</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531498028055736</v>
+        <v>4.531448717224751</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550340783256731</v>
+        <v>4.550290466818294</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582710373017675</v>
+        <v>4.582653818756863</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601013692742358</v>
+        <v>4.600941299549605</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673399516783292</v>
+        <v>4.673316496314477</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708890284902091</v>
+        <v>4.708802245215725</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775713439333154</v>
+        <v>4.775630186783939</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812037208706917</v>
+        <v>4.811988384025145</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809814090255863</v>
+        <v>4.809766207832275</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819021578982753</v>
+        <v>4.818973636726311</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862248186941123</v>
+        <v>4.862243270463164</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855034769191637</v>
+        <v>4.855031863343399</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853443315593273</v>
+        <v>4.853465469730587</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830478506370953</v>
+        <v>4.830494263014311</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838443197992547</v>
+        <v>4.838464025390882</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891772511994999</v>
+        <v>4.891809535441361</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918063593378326</v>
+        <v>4.918085537543922</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927289642193898</v>
+        <v>4.927311929320361</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917389238893117</v>
+        <v>4.917411066516673</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898154078609513</v>
+        <v>4.898171585865719</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896691321848115</v>
+        <v>4.89672075409726</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897574123238543</v>
+        <v>4.897615558122583</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895179109891517</v>
+        <v>4.895234089889127</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879710476913154</v>
+        <v>4.879767032737919</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856185974963108</v>
+        <v>4.856233476523716</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829900237783347</v>
+        <v>4.829945402633699</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820606947669816</v>
+        <v>4.820649981045802</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790435962539044</v>
+        <v>4.79047174566028</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762500782814383</v>
+        <v>4.762537188471093</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751602192898297</v>
+        <v>4.751639330150703</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756190969411519</v>
+        <v>4.756250411423604</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750646294114738</v>
+        <v>4.750683751009201</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750437789023433</v>
+        <v>4.750445468113478</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755487659356472</v>
+        <v>4.755454998704582</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759870121769653</v>
+        <v>4.759780304163439</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.7673187804197</v>
+        <v>4.767180414429511</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.773718762530776</v>
+        <v>4.773553118162328</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.771442843778392</v>
+        <v>4.77127504277378</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.76429031139006</v>
+        <v>4.764167097743536</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.759035310298966</v>
+        <v>4.757060874649518</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.758079991281928</v>
+        <v>4.755807813528454</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.760144146063579</v>
+        <v>4.757705626636485</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.774141695957262</v>
+        <v>4.770638967000911</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.781248137964169</v>
+        <v>4.77715488624871</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.784391753348382</v>
+        <v>4.779696969499332</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.777200975948514</v>
+        <v>4.771786704519649</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.774083153275956</v>
+        <v>4.767518500819975</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.754467288394627</v>
+        <v>4.746971365224946</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.725740808837029</v>
+        <v>4.716709062378694</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.667922576908365</v>
+        <v>4.658191502377445</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.583390020847558</v>
+        <v>4.574389160901308</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.526178570867562</v>
+        <v>4.514829716440479</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.462211070867562</v>
+        <v>4.450862216440479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-01_20-38-33
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.757060874649518</v>
+        <v>4.756403558632273</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.755807813528454</v>
+        <v>4.755071458200127</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.757705626636485</v>
+        <v>4.756901379537625</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.770638967000911</v>
+        <v>4.770031721874261</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.77715488624871</v>
+        <v>4.776385418126864</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.779696969499332</v>
+        <v>4.77878288613497</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.771786704519649</v>
+        <v>4.770694031630211</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.767518500819975</v>
+        <v>4.766221142175699</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.746971365224946</v>
+        <v>4.745424682591651</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.716709062378694</v>
+        <v>4.714814072773732</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.658191502377445</v>
+        <v>4.65567534372574</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.574389160901308</v>
+        <v>4.570811173603128</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.514829716440479</v>
+        <v>4.509122847880995</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.450862216440479</v>
+        <v>4.444322847880995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-02_20-38-58
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712814855230546</v>
+        <v>4.712814269033649</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711764459791539</v>
+        <v>4.711767186648236</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720300377105684</v>
+        <v>4.720303727537225</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707174599758295</v>
+        <v>4.707181515629655</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694524033591122</v>
+        <v>4.694531028273309</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678601018838553</v>
+        <v>4.678608074299672</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673610722438372</v>
+        <v>4.673617796614664</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68668686029552</v>
+        <v>4.686693936451657</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702684504390717</v>
+        <v>4.702693033865096</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705794417055547</v>
+        <v>4.705800084292882</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694868956951511</v>
+        <v>4.694874733675253</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664914056803559</v>
+        <v>4.664920310657695</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649679657885559</v>
+        <v>4.649680699362919</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641456081291172</v>
+        <v>4.641458477406712</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636265312856521</v>
+        <v>4.636266775915233</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634084358595198</v>
+        <v>4.634087804763289</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637408074823274</v>
+        <v>4.637408962458743</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634386689025769</v>
+        <v>4.634384787524121</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627431498818609</v>
+        <v>4.627425734204615</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623679589523932</v>
+        <v>4.623673437937958</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599041639916377</v>
+        <v>4.599035586848247</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579231144034479</v>
+        <v>4.579218285514024</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560252975693226</v>
+        <v>4.560232246057661</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521983166017675</v>
+        <v>4.521952456981483</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518753145888986</v>
+        <v>4.518709458318451</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531448717224751</v>
+        <v>4.531400281145297</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550290466818294</v>
+        <v>4.550241040227914</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582653818756863</v>
+        <v>4.582598260420736</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600941299549605</v>
+        <v>4.600870163145766</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673316496314477</v>
+        <v>4.673234918948378</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708802245215725</v>
+        <v>4.708715736305664</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775630186783939</v>
+        <v>4.77554836086458</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811988384025145</v>
+        <v>4.81194039762962</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809766207832275</v>
+        <v>4.809719143000642</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818973636726311</v>
+        <v>4.818926507386143</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862243270463164</v>
+        <v>4.862238432179074</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855031863343399</v>
+        <v>4.855028999969074</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853465469730587</v>
+        <v>4.853487239555461</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830494263014311</v>
+        <v>4.830509739839844</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838464025390882</v>
+        <v>4.838484486272402</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891809535441361</v>
+        <v>4.891845913438749</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918085537543922</v>
+        <v>4.918107088410379</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927311929320361</v>
+        <v>4.927333818626405</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917411066516673</v>
+        <v>4.917432514456398</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898171585865719</v>
+        <v>4.898188786795695</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89672075409726</v>
+        <v>4.896749680586435</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897615558122583</v>
+        <v>4.897656290817004</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895234089889127</v>
+        <v>4.895288132209057</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879767032737919</v>
+        <v>4.879822621752089</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856233476523716</v>
+        <v>4.856280159218379</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829945402633699</v>
+        <v>4.829989776319476</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820649981045802</v>
+        <v>4.820692257586662</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.79047174566028</v>
+        <v>4.790506886701917</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762537188471093</v>
+        <v>4.762572952601124</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751639330150703</v>
+        <v>4.75167583151173</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756250411423604</v>
+        <v>4.75630889476934</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750683751009201</v>
+        <v>4.750720665982707</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750445468113478</v>
+        <v>4.750453126081053</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755454998704582</v>
+        <v>4.755423009350965</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759780304163439</v>
+        <v>4.759692072132168</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.767180414429511</v>
+        <v>4.767044357822463</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.773553118162328</v>
+        <v>4.773390135920712</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.77127504277378</v>
+        <v>4.771109720872651</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.764167097743536</v>
+        <v>4.76404536665116</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.756403558632273</v>
+        <v>4.753727364554747</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.755071458200127</v>
+        <v>4.752008161692649</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.756901379537625</v>
+        <v>4.753573204435877</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.770031721874261</v>
+        <v>4.765861318545101</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.776385418126864</v>
+        <v>4.771482660422143</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.77878288613497</v>
+        <v>4.77315519731448</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.770694031630211</v>
+        <v>4.764198473940219</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.766221142175699</v>
+        <v>4.758433581160877</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.745424682591651</v>
+        <v>4.736530066728029</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.714814072773732</v>
+        <v>4.70417823257576</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.65567534372574</v>
+        <v>4.643935860807323</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.570811173603128</v>
+        <v>4.558982272894545</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.509122847880995</v>
+        <v>4.49420563988242</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.444322847880995</v>
+        <v>4.386687261136367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-03_09-31-02
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712814269033649</v>
+        <v>4.712813693030702</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711767186648236</v>
+        <v>4.711769865883791</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720303727537225</v>
+        <v>4.72030701976484</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707181515629655</v>
+        <v>4.707188311112884</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694531028273309</v>
+        <v>4.694537901200106</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678608074299672</v>
+        <v>4.678615006947107</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673617796614664</v>
+        <v>4.673624747678891</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686693936451657</v>
+        <v>4.686700889534536</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702693033865096</v>
+        <v>4.702701415485345</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705800084292882</v>
+        <v>4.70580565341291</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694874733675253</v>
+        <v>4.694880410343435</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664920310657695</v>
+        <v>4.664926456106187</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649680699362919</v>
+        <v>4.649681724794124</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641458477406712</v>
+        <v>4.641460833564159</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636266775915233</v>
+        <v>4.636268213603722</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634087804763289</v>
+        <v>4.634091191472189</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637408962458743</v>
+        <v>4.637409836089285</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634384787524121</v>
+        <v>4.634382919491163</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627425734204615</v>
+        <v>4.627420069109787</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623673437937958</v>
+        <v>4.623667392839967</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599035586848247</v>
+        <v>4.599029638846872</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579218285514024</v>
+        <v>4.579205654214396</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560232246057661</v>
+        <v>4.560211884656659</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521952456981483</v>
+        <v>4.52192229115653</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518709458318451</v>
+        <v>4.518666541907528</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531400281145297</v>
+        <v>4.531352696774569</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550241040227914</v>
+        <v>4.550192480121452</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582598260420736</v>
+        <v>4.582543671975492</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600870163145766</v>
+        <v>4.600800251118386</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673234918948378</v>
+        <v>4.673154747422894</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708715736305664</v>
+        <v>4.708630718634591</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.77554836086458</v>
+        <v>4.775467925260077</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81194039762962</v>
+        <v>4.811893228141504</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809719143000642</v>
+        <v>4.809672875029392</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818926507386143</v>
+        <v>4.818880170501069</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862238432179074</v>
+        <v>4.862233670256672</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855028999969074</v>
+        <v>4.855026178178032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853487239555461</v>
+        <v>4.853508634977461</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830509739839844</v>
+        <v>4.830524944230213</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838484486272402</v>
+        <v>4.838504590218641</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891845913438749</v>
+        <v>4.891881662713141</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918107088410379</v>
+        <v>4.918128256436143</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927333818626405</v>
+        <v>4.927355320645154</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917432514456398</v>
+        <v>4.917453592514326</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898188786795695</v>
+        <v>4.898205689348869</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896749680586435</v>
+        <v>4.896778114216764</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897656290817004</v>
+        <v>4.897696338982396</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895288132209057</v>
+        <v>4.895341260592915</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879822621752089</v>
+        <v>4.879877268503938</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856280159218379</v>
+        <v>4.856326044022818</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829989776319476</v>
+        <v>4.830033379434274</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820692257586662</v>
+        <v>4.820733797072549</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790506886701917</v>
+        <v>4.790541402755333</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762572952601124</v>
+        <v>4.762608091934513</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.75167583151173</v>
+        <v>4.751711713060969</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75630889476934</v>
+        <v>4.75636644221877</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750720665982707</v>
+        <v>4.750757050231963</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750453126081053</v>
+        <v>4.75046076075277</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755423009350965</v>
+        <v>4.755391671694648</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759692072132168</v>
+        <v>4.759605384781538</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.767044357822463</v>
+        <v>4.766910554427024</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.773390135920712</v>
+        <v>4.773229753991858</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.771109720872651</v>
+        <v>4.770946826540115</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.76404536665116</v>
+        <v>4.763925096976578</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.753727364554747</v>
+        <v>4.751159402103559</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.752008161692649</v>
+        <v>4.749065189980271</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.753573204435877</v>
+        <v>4.750384617127056</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.765861318545101</v>
+        <v>4.761865382291184</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.771482660422143</v>
+        <v>4.766800328431695</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.77315519731448</v>
+        <v>4.767794340807061</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.764198473940219</v>
+        <v>4.758038951415065</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.758433581160877</v>
+        <v>4.751092163359269</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.736530066728029</v>
+        <v>4.728215978578129</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.70417823257576</v>
+        <v>4.69436109255598</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.643935860807323</v>
+        <v>4.63336996443858</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.558982272894545</v>
+        <v>4.54878194259312</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.49420563988242</v>
+        <v>4.482328198033335</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.386687261136367</v>
+        <v>4.375651998105295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-04_19-59-47
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712813693030702</v>
+        <v>4.712813126958096</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711769865883791</v>
+        <v>4.711772498734784</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.72030701976484</v>
+        <v>4.720310255291981</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707188311112884</v>
+        <v>4.70719498932394</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694537901200106</v>
+        <v>4.694544655522751</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678615006947107</v>
+        <v>4.678621819959497</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673624747678891</v>
+        <v>4.67363157881671</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686700889534536</v>
+        <v>4.686707722726924</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702701415485345</v>
+        <v>4.702709653062115</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70580565341291</v>
+        <v>4.705811126941495</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694880410343435</v>
+        <v>4.694885989532919</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664926456106187</v>
+        <v>4.664932495943156</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649681724794124</v>
+        <v>4.649682734540971</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641460833564159</v>
+        <v>4.641463150753053</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636268213603722</v>
+        <v>4.636269626576242</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634091191472189</v>
+        <v>4.634094520247046</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637409836089285</v>
+        <v>4.63741069604009</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634382919491163</v>
+        <v>4.634381084051707</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627420069109787</v>
+        <v>4.627414500979974</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623667392839967</v>
+        <v>4.623661451489088</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599029638846872</v>
+        <v>4.599023793201251</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579205654214396</v>
+        <v>4.579193244169461</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560211884656659</v>
+        <v>4.56019188177477</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.52192229115653</v>
+        <v>4.521892654270901</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518666541907528</v>
+        <v>4.518624376438687</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531352696774569</v>
+        <v>4.531305941871068</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550192480121452</v>
+        <v>4.550144763944457</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582543671975492</v>
+        <v>4.582490028285381</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600800251118386</v>
+        <v>4.600731532158907</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673154747422894</v>
+        <v>4.673075945746443</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708630718634591</v>
+        <v>4.708547154013685</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775467925260077</v>
+        <v>4.77538884487609</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811893228141504</v>
+        <v>4.811846854901894</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809672875029392</v>
+        <v>4.809627383880898</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818880170501069</v>
+        <v>4.818834606289467</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862233670256672</v>
+        <v>4.862228982919889</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855026178178032</v>
+        <v>4.855023397103015</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853508634977461</v>
+        <v>4.853529665568512</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830524944230213</v>
+        <v>4.830539883310819</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838504590218641</v>
+        <v>4.838524346480338</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891881662713141</v>
+        <v>4.891916799417784</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918128256436143</v>
+        <v>4.918149051712811</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927355320645154</v>
+        <v>4.92737644554194</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917453592514326</v>
+        <v>4.917474310158639</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898205689348869</v>
+        <v>4.89822230120266</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896778114216764</v>
+        <v>4.896806067455119</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897696338982396</v>
+        <v>4.897735719693388</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895341260592915</v>
+        <v>4.895393497988993</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879877268503938</v>
+        <v>4.879930996718755</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856326044022818</v>
+        <v>4.856371151203009</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.830033379434274</v>
+        <v>4.830076231863618</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820733797072549</v>
+        <v>4.820774618600685</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790541402755333</v>
+        <v>4.790575310311875</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762608091934513</v>
+        <v>4.762642622627228</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751711713060969</v>
+        <v>4.751746990344282</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75636644221877</v>
+        <v>4.75642307583486</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750757050231963</v>
+        <v>4.750792914665945</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.75046076075277</v>
+        <v>4.750468370115285</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755391671694648</v>
+        <v>4.755360966866185</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759605384781538</v>
+        <v>4.759520202588098</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.766910554427024</v>
+        <v>4.766778949839081</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.773229753991858</v>
+        <v>4.773071912396</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.770946826540115</v>
+        <v>4.770786309545969</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.763925096976578</v>
+        <v>4.763806267731916</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.751159402103559</v>
+        <v>4.748962413756845</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.749065189980271</v>
+        <v>4.746544984643587</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.750384617127056</v>
+        <v>4.747710422236904</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.761865382291184</v>
+        <v>4.758443355937899</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.766800328431695</v>
+        <v>4.762769367097919</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.767794340807061</v>
+        <v>4.763167042329309</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.758038951415065</v>
+        <v>4.752740953556224</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.751092163359269</v>
+        <v>4.744796700088827</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.728215978578129</v>
+        <v>4.721178578456881</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.69436109255598</v>
+        <v>4.686229005565752</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.63336996443858</v>
+        <v>4.625067325664327</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.54878194259312</v>
+        <v>4.541627171692357</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.482328198033335</v>
+        <v>4.475190469642675</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.375651998105295</v>
+        <v>4.374667454700552</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-05_20-37-45
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712813126958096</v>
+        <v>4.712812570561233</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711772498734784</v>
+        <v>4.711775086395358</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720310255291981</v>
+        <v>4.720313435570768</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70719498932394</v>
+        <v>4.707201553272184</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694544655522751</v>
+        <v>4.694551294284682</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678621819959497</v>
+        <v>4.678628516406747</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67363157881671</v>
+        <v>4.673638293104828</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686707722726924</v>
+        <v>4.686714439102799</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702709653062115</v>
+        <v>4.702717750276245</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705811126941495</v>
+        <v>4.705816507318547</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694885989532919</v>
+        <v>4.694891473732842</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664932495943156</v>
+        <v>4.664938432867531</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649682734540971</v>
+        <v>4.649683728954694</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641463150753053</v>
+        <v>4.641465429930589</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636269626576242</v>
+        <v>4.63627101546474</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634094520247046</v>
+        <v>4.634097792561303</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63741069604009</v>
+        <v>4.637411542626491</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634381084051707</v>
+        <v>4.634379280360796</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627414500979974</v>
+        <v>4.627409027347653</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623661451489088</v>
+        <v>4.623655611237697</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599023793201251</v>
+        <v>4.599018047292819</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579193244169461</v>
+        <v>4.579181049620007</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.56019188177477</v>
+        <v>4.56017222803501</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521892654270901</v>
+        <v>4.5218635325478</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518624376438687</v>
+        <v>4.518582942394259</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531305941871068</v>
+        <v>4.531259994960119</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550144763944457</v>
+        <v>4.550097869917447</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582490028285381</v>
+        <v>4.582437305074386</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600731532158907</v>
+        <v>4.600663976016122</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673075945746443</v>
+        <v>4.67299847914433</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708547154013685</v>
+        <v>4.708465005545679</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.77538884487609</v>
+        <v>4.775311085788147</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811846854901894</v>
+        <v>4.811801257941799</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809627383880898</v>
+        <v>4.809582650182746</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818834606289467</v>
+        <v>4.818789795621351</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862228982919889</v>
+        <v>4.862224368446669</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855023397103015</v>
+        <v>4.855020655899454</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853529665568512</v>
+        <v>4.853550340577163</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830539883310819</v>
+        <v>4.830554563960907</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838524346480338</v>
+        <v>4.838543763991593</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891916799417784</v>
+        <v>4.891951339157499</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918149051712811</v>
+        <v>4.918169483981044</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.92737644554194</v>
+        <v>4.927397203130183</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917474310158639</v>
+        <v>4.91749467653771</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89822230120266</v>
+        <v>4.898238629773989</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896806067455119</v>
+        <v>4.896833552352193</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897735719693388</v>
+        <v>4.897774449462693</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895393497988993</v>
+        <v>4.895444866585073</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879930996718755</v>
+        <v>4.879983829332986</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856371151203009</v>
+        <v>4.856415500344924</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.830076231863618</v>
+        <v>4.830118352815111</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820774618600685</v>
+        <v>4.820814740614582</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790575310311875</v>
+        <v>4.7906086252889</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762642622627228</v>
+        <v>4.762676560285465</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751746990344282</v>
+        <v>4.751781678395606</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75642307583486</v>
+        <v>4.756478817000367</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750792914665945</v>
+        <v>4.750828269914162</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750468370115285</v>
+        <v>4.750475952305218</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755360966866185</v>
+        <v>4.755330876694717</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759520202588098</v>
+        <v>4.759436487343239</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.766778949839081</v>
+        <v>4.766649491354659</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.773071912396</v>
+        <v>4.772916552923015</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.770786309545969</v>
+        <v>4.770628120929301</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.763806267731916</v>
+        <v>4.763688858094497</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.748962413756845</v>
+        <v>4.746851997301583</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.746544984643587</v>
+        <v>4.744116151667037</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.747710422236904</v>
+        <v>4.745138581639746</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.758443355937899</v>
+        <v>4.755152208039977</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.762769367097919</v>
+        <v>4.758893733887946</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.763167042329309</v>
+        <v>4.758726439074216</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.752740953556224</v>
+        <v>4.747675431008058</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.744796700088827</v>
+        <v>4.738807925743501</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.721178578456881</v>
+        <v>4.71452973356757</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.686229005565752</v>
+        <v>4.678639402264116</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.625067325664327</v>
+        <v>4.617468439669945</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.541627171692357</v>
+        <v>4.53527066806268</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.475190469642675</v>
+        <v>4.469171041563716</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.374667454700552</v>
+        <v>4.37385517501132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-07_20-54-42
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.743385057786005</v>
+        <v>4.74339024386127</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.752951007028947</v>
+        <v>4.752943432164209</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.755925610986514</v>
+        <v>4.756104680472498</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.755410721349078</v>
+        <v>4.755550826386737</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.743981070785473</v>
+        <v>4.744077493833107</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.734503009480263</v>
+        <v>4.734566755919614</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.709938077737332</v>
+        <v>4.709975948037088</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.674068992078551</v>
+        <v>4.674084996481527</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.613148521834317</v>
+        <v>4.613150779928613</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.53295098335251</v>
+        <v>4.532933705803619</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.468237335254965</v>
+        <v>4.468203679790937</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.379874735680179</v>
+        <v>4.379812135037787</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.374684952324732</v>
+        <v>4.374251462507771</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-08_20-37-38
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712812023594141</v>
+        <v>4.712811485819119</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711777630019017</v>
+        <v>4.711780130720337</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720316562004165</v>
+        <v>4.72031963594803</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707208005864893</v>
+        <v>4.707214349911563</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694557820426097</v>
+        <v>4.69456423678831</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678635099254626</v>
+        <v>4.678641571369154</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673644893515607</v>
+        <v>4.673651382921459</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686721041631946</v>
+        <v>4.68672753318435</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702725710684245</v>
+        <v>4.702733537723506</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705821796901652</v>
+        <v>4.70582699796952</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694896865348318</v>
+        <v>4.694902166703958</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664944269487067</v>
+        <v>4.66495000832216</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649684708376338</v>
+        <v>4.649685673137119</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641467672022919</v>
+        <v>4.641469877926403</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636272380879801</v>
+        <v>4.636273723411541</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634101009838883</v>
+        <v>4.634104173456235</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63741237615433</v>
+        <v>4.637413196920313</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634377507602404</v>
+        <v>4.634375764988212</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627403645828299</v>
+        <v>4.627398354116909</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623649869527487</v>
+        <v>4.623644223885726</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599012398591548</v>
+        <v>4.59900684465223</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579169065004866</v>
+        <v>4.579157284952474</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560152914384267</v>
+        <v>4.560133932079443</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521834912684293</v>
+        <v>4.521806781831115</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518542220926452</v>
+        <v>4.518502193828883</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531214835301135</v>
+        <v>4.531170442856559</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550051777002945</v>
+        <v>4.550006464874195</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.58238547888982</v>
+        <v>4.582334527067781</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600597553451956</v>
+        <v>4.600532236199448</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.672922314007796</v>
+        <v>4.672847417845619</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708384237570776</v>
+        <v>4.708304815615257</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775234615193359</v>
+        <v>4.775159401364506</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811756417953616</v>
+        <v>4.811712316264011</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809538655200391</v>
+        <v>4.809495380811164</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818745719991821</v>
+        <v>4.818702361495784</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862219825166958</v>
+        <v>4.862215351460792</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855017953744784</v>
+        <v>4.855015289837803</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853570668942104</v>
+        <v>4.853590659305045</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830568992824087</v>
+        <v>4.830583176318347</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83856285138327</v>
+        <v>4.838581616995759</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891985297011749</v>
+        <v>4.892018687556546</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918189562645669</v>
+        <v>4.91820929679</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927417602886461</v>
+        <v>4.927437653964807</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917514700493485</v>
+        <v>4.917534390574168</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898254682230204</v>
+        <v>4.898270465499468</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896860580559702</v>
+        <v>4.896887163346721</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.89781254426398</v>
+        <v>4.897850019553639</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895495387839605</v>
+        <v>4.895545082511381</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.880035788526714</v>
+        <v>4.880086895754538</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856459110382782</v>
+        <v>4.856501999625927</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.830159760847052</v>
+        <v>4.830200473895629</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820854180931748</v>
+        <v>4.82089295677001</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790641363054501</v>
+        <v>4.79067353845093</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762709919988735</v>
+        <v>4.762742716311801</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751815791757691</v>
+        <v>4.751849344501863</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756533686443507</v>
+        <v>4.756587704262485</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750863126334673</v>
+        <v>4.750897494021901</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750483505599735</v>
+        <v>4.750491028407724</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755301383676731</v>
+        <v>4.755272470946484</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759354202099867</v>
+        <v>4.759273311121602</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.766522127905623</v>
+        <v>4.766396809998165</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.772763619070329</v>
+        <v>4.77261305598326</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.770472212963909</v>
+        <v>4.770318539124492</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.763572847421658</v>
+        <v>4.763458215263835</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.746800069252162</v>
+        <v>4.746748299683611</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.742537456461065</v>
+        <v>4.740779350583887</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.74339024386127</v>
+        <v>4.74142752731998</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.752943432164209</v>
+        <v>4.750470495532197</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.756104680472498</v>
+        <v>4.753054114198476</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.755550826386737</v>
+        <v>4.752096231279593</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.744077493833107</v>
+        <v>4.740184421913841</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.734566755919614</v>
+        <v>4.730024973138567</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.709975948037088</v>
+        <v>4.705101164441701</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.674084996481527</v>
+        <v>4.669169795238999</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.613150779928613</v>
+        <v>4.608392961529107</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.532933705803619</v>
+        <v>4.529890729472869</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.468203679790937</v>
+        <v>4.466222075645955</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.379812135037787</v>
+        <v>4.382529506816095</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.374251462507771</v>
+        <v>4.368186415808998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-09_20-33-27
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712811485819119</v>
+        <v>4.712816677764813</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711780130720337</v>
+        <v>4.711755980451395</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.72031963594803</v>
+        <v>4.720289960734035</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707214349911563</v>
+        <v>4.707153096955049</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.69456423678831</v>
+        <v>4.694502285779874</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678641571369154</v>
+        <v>4.678579082051701</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673651382921459</v>
+        <v>4.673588727642117</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68672753318435</v>
+        <v>4.686664859824165</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702733537723506</v>
+        <v>4.702657988665831</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70582699796952</v>
+        <v>4.705776800010221</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694902166703958</v>
+        <v>4.694850999279153</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.66495000832216</v>
+        <v>4.664894615347644</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649685673137119</v>
+        <v>4.649676433391994</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641469877926403</v>
+        <v>4.641448642786033</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636273723411541</v>
+        <v>4.636260764560724</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634104173456235</v>
+        <v>4.634073647259902</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637413196920313</v>
+        <v>4.637405324479514</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634375764988212</v>
+        <v>4.634392603577212</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627398354116909</v>
+        <v>4.627449416698511</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623644223885726</v>
+        <v>4.623698712105675</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59900684465223</v>
+        <v>4.599060458105832</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579157284952474</v>
+        <v>4.579271145886548</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560133932079443</v>
+        <v>4.560317476568055</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521806781831115</v>
+        <v>4.52207870301923</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518502193828883</v>
+        <v>4.518889048907768</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531170442856559</v>
+        <v>4.531599370370278</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550006464874195</v>
+        <v>4.550444183404426</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582334527067781</v>
+        <v>4.582826578183428</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600532236199448</v>
+        <v>4.601162384960733</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.672847417845619</v>
+        <v>4.673570042772052</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708304815615257</v>
+        <v>4.70907112185864</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775159401364506</v>
+        <v>4.775884376008118</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811712316264011</v>
+        <v>4.812137462235389</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809495380811164</v>
+        <v>4.809912394458091</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818702361495784</v>
+        <v>4.81911998766468</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862215351460792</v>
+        <v>4.86225826210123</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855015289837803</v>
+        <v>4.855040711993553</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853590659305045</v>
+        <v>4.853397812963987</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830583176318347</v>
+        <v>4.830446122742938</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838581616995759</v>
+        <v>4.838400403575134</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.892018687556546</v>
+        <v>4.891696458832852</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.91820929679</v>
+        <v>4.918018481380027</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927437653964807</v>
+        <v>4.927243830406889</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917534390574168</v>
+        <v>4.917344403627334</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898270465499468</v>
+        <v>4.898118111887308</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896887163346721</v>
+        <v>4.896630886178917</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897850019553639</v>
+        <v>4.897489073176394</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895545082511381</v>
+        <v>4.895066237721409</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.880086895754538</v>
+        <v>4.879594362306189</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856501999625927</v>
+        <v>4.856088427602831</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.830200473895629</v>
+        <v>4.829807448481734</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.82089295677001</v>
+        <v>4.820518527690888</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.79067353845093</v>
+        <v>4.790362398525678</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762742716311801</v>
+        <v>4.762425976975427</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751849344501863</v>
+        <v>4.754124074269</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756587704262485</v>
+        <v>4.756006653768317</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750897494021901</v>
+        <v>4.749307701444614</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750491028407724</v>
+        <v>4.746764994045649</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755272470946484</v>
+        <v>4.749918451376509</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759273311121602</v>
+        <v>4.751793173863797</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.766396809998165</v>
+        <v>4.75489735621687</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.77261305598326</v>
+        <v>4.76152090868796</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.770318539124492</v>
+        <v>4.759487114728357</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.763458215263835</v>
+        <v>4.753577634963321</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.746748299683611</v>
+        <v>4.738501355463036</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.740779350583887</v>
+        <v>4.727357177942613</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.74142752731998</v>
+        <v>4.727776559681331</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.750470495532197</v>
+        <v>4.741037591805286</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.753054114198476</v>
+        <v>4.741779496271077</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.752096231279593</v>
+        <v>4.744590539878175</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.740184421913841</v>
+        <v>4.73930688773696</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.730024973138567</v>
+        <v>4.725791879271162</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.705101164441701</v>
+        <v>4.698733384196634</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.669169795238999</v>
+        <v>4.659630332769</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.608392961529107</v>
+        <v>4.615980314033138</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.529890729472869</v>
+        <v>4.535486714076201</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.466222075645955</v>
+        <v>4.470495524437002</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.382529506816095</v>
+        <v>4.394942406060663</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.368186415808998</v>
+        <v>4.400585808373822</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-10_10-10-49
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712816677764813</v>
+        <v>4.712810436933758</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711755980451395</v>
+        <v>4.711785007629333</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720289960734035</v>
+        <v>4.720325631566793</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707153096955049</v>
+        <v>4.707226723140066</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694502285779874</v>
+        <v>4.694576751070436</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678579082051701</v>
+        <v>4.678654194388205</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673588727642117</v>
+        <v>4.673664039733055</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686664859824165</v>
+        <v>4.686740194364547</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702657988665831</v>
+        <v>4.702748804879173</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705776800010221</v>
+        <v>4.705837143299406</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694850999279153</v>
+        <v>4.694912507551509</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664894615347644</v>
+        <v>4.664961202305395</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649676433391994</v>
+        <v>4.649687559953829</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641448642786033</v>
+        <v>4.641474184610382</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636260764560724</v>
+        <v>4.636276342088258</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634073647259902</v>
+        <v>4.634110344990403</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637405324479514</v>
+        <v>4.637414801309792</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634392603577212</v>
+        <v>4.634372367170747</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627449416698511</v>
+        <v>4.627388031276121</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623698712105675</v>
+        <v>4.623633211323429</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599060458105832</v>
+        <v>4.598996011681783</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579271145886548</v>
+        <v>4.579134317950068</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560317476568055</v>
+        <v>4.560096928007053</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.52207870301923</v>
+        <v>4.521751937913112</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518889048907768</v>
+        <v>4.518424152965123</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531599370370278</v>
+        <v>4.53108388279996</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550444183404426</v>
+        <v>4.549918105043642</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582826578183428</v>
+        <v>4.582235159604195</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601162384960733</v>
+        <v>4.600404809179402</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673570042772052</v>
+        <v>4.672701307793228</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.70907112185864</v>
+        <v>4.708149877507116</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775884376008118</v>
+        <v>4.775012622214086</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812137462235389</v>
+        <v>4.811626256104966</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809912394458091</v>
+        <v>4.809410924233523</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.81911998766468</v>
+        <v>4.818617727139658</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86225826210123</v>
+        <v>4.862206606528675</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855040711993553</v>
+        <v>4.855010073665101</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853397812963987</v>
+        <v>4.853629659179598</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830446122742938</v>
+        <v>4.830610831800363</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838400403575134</v>
+        <v>4.83861821486436</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891696458832852</v>
+        <v>4.89208382262858</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918018481380027</v>
+        <v>4.918247766324377</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927243830406889</v>
+        <v>4.927476745171937</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917344403627334</v>
+        <v>4.917572801906271</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898118111887308</v>
+        <v>4.898301251052603</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896630886178917</v>
+        <v>4.896939035914965</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897489073176394</v>
+        <v>4.897923170960617</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895066237721409</v>
+        <v>4.895642071811571</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879594362306189</v>
+        <v>4.880186636678346</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856088427602831</v>
+        <v>4.856585685993074</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829807448481734</v>
+        <v>4.830279883830615</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820518527690888</v>
+        <v>4.820968581031511</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790362398525678</v>
+        <v>4.790736259008595</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762425976975427</v>
+        <v>4.762806674716734</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.754124074269</v>
+        <v>4.751914822176648</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756006653768317</v>
+        <v>4.756693262410423</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749307701444614</v>
+        <v>4.750964802301307</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746764994045649</v>
+        <v>4.750505976809409</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.749918451376509</v>
+        <v>4.755216321908033</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.751793173863797</v>
+        <v>4.759115574780293</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.75489735621687</v>
+        <v>4.766152120354065</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.76152090868796</v>
+        <v>4.772318830585212</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.759487114728357</v>
+        <v>4.770017713529723</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.753577634963321</v>
+        <v>4.763233005727929</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.738501355463036</v>
+        <v>4.746645285910866</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.727357177942613</v>
+        <v>4.737361035880289</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.727776559681331</v>
+        <v>4.73762527333687</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.741037591805286</v>
+        <v>4.745630327106086</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.741779496271077</v>
+        <v>4.747100445834832</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.744590539878175</v>
+        <v>4.745420711542181</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.73930688773696</v>
+        <v>4.732688752330866</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.725791879271162</v>
+        <v>4.721326227672531</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.698733384196634</v>
+        <v>4.69579672047006</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.659630332769</v>
+        <v>4.659804651328164</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.615980314033138</v>
+        <v>4.599308754912077</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.535486714076201</v>
+        <v>4.523759969225043</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.470495524437002</v>
+        <v>4.461695451314686</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.394942406060663</v>
+        <v>4.384115309638053</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.400585808373822</v>
+        <v>4.35938022019532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-12_20-33-49
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712810436933758</v>
+        <v>4.712816059308125</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711785007629333</v>
+        <v>4.711758858044636</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720325631566793</v>
+        <v>4.720293495346483</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707226723140066</v>
+        <v>4.707160393825526</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694576751070436</v>
+        <v>4.694509665787476</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678654194388205</v>
+        <v>4.678586526187582</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673664039733055</v>
+        <v>4.67359619143271</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686740194364547</v>
+        <v>4.686672325459038</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702748804879173</v>
+        <v>4.702666985953012</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705837143299406</v>
+        <v>4.705782777672652</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694912507551509</v>
+        <v>4.694857092567699</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664961202305395</v>
+        <v>4.66490121220027</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649687559953829</v>
+        <v>4.649677525290071</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641474184610382</v>
+        <v>4.641451165057606</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636276342088258</v>
+        <v>4.636262307893886</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634110344990403</v>
+        <v>4.634077281508503</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637414801309792</v>
+        <v>4.637406256185238</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634372367170747</v>
+        <v>4.634390596095246</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627388031276121</v>
+        <v>4.627443337277058</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623633211323429</v>
+        <v>4.62369222361461</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.598996011681783</v>
+        <v>4.599054072584001</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579134317950068</v>
+        <v>4.579257567693807</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560096928007053</v>
+        <v>4.560295580315382</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521751937913112</v>
+        <v>4.522046273422818</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518424152965123</v>
+        <v>4.518842919069789</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.53108388279996</v>
+        <v>4.531548237518736</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.549918105043642</v>
+        <v>4.55039201375366</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582235159604195</v>
+        <v>4.582767950175429</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600404809179402</v>
+        <v>4.60108737628941</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.672701307793228</v>
+        <v>4.673484018943933</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708149877507116</v>
+        <v>4.70897989631057</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775012622214086</v>
+        <v>4.775798156101363</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811626256104966</v>
+        <v>4.812086893805286</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809410924233523</v>
+        <v>4.809862811727189</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818617727139658</v>
+        <v>4.819070355325569</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862206606528675</v>
+        <v>4.862253183503444</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855010073665101</v>
+        <v>4.855037718428507</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853629659179598</v>
+        <v>4.853420766881301</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830610831800363</v>
+        <v>4.830462462258145</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83861821486436</v>
+        <v>4.838421994150176</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.89208382262858</v>
+        <v>4.891734825775365</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918247766324377</v>
+        <v>4.918041245071505</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927476745171937</v>
+        <v>4.927266946329362</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917572801906271</v>
+        <v>4.917367021435004</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898301251052603</v>
+        <v>4.898136256793526</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896939035914965</v>
+        <v>4.896661370484582</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897923170960617</v>
+        <v>4.897531967893042</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895642071811571</v>
+        <v>4.8951231676468</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.880186636678346</v>
+        <v>4.879652928870575</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856585685993074</v>
+        <v>4.856137632819761</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.830279883830615</v>
+        <v>4.829854260434959</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820968581031511</v>
+        <v>4.820563136964852</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790736259008595</v>
+        <v>4.790399519619315</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762806674716734</v>
+        <v>4.76246371830128</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751914822176648</v>
+        <v>4.754161082569833</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756693262410423</v>
+        <v>4.756070390823817</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750964802301307</v>
+        <v>4.749351625754665</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750505976809409</v>
+        <v>4.746783366000766</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755216321908033</v>
+        <v>4.749898471482578</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759115574780293</v>
+        <v>4.751714646796709</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.766152120354065</v>
+        <v>4.754771157079228</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.772318830585212</v>
+        <v>4.761361447439354</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.770017713529723</v>
+        <v>4.75931715062923</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.763233005727929</v>
+        <v>4.753434924081958</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.746645285910866</v>
+        <v>4.73840884947211</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.737361035880289</v>
+        <v>4.726029704351049</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.73762527333687</v>
+        <v>4.726152688549943</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.745630327106086</v>
+        <v>4.739074832150575</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.747100445834832</v>
+        <v>4.738960076408929</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.745420711542181</v>
+        <v>4.741526044559249</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.732688752330866</v>
+        <v>4.73565068798594</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.721326227672531</v>
+        <v>4.72167422113746</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.69579672047006</v>
+        <v>4.694505389633514</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.659804651328164</v>
+        <v>4.655872121761959</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.599308754912077</v>
+        <v>4.612562565041443</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.523759969225043</v>
+        <v>4.534758397774175</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.461695451314686</v>
+        <v>4.472037576596928</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.384115309638053</v>
+        <v>4.401364474041877</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.35938022019532</v>
+        <v>4.405114655033812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-12_20-37-50
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712816059308125</v>
+        <v>4.712809925386333</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711758858044636</v>
+        <v>4.711787385885795</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720293495346483</v>
+        <v>4.72032855573508</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707160393825526</v>
+        <v>4.707232757487633</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694509665787476</v>
+        <v>4.694582854214598</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678586526187582</v>
+        <v>4.678660350562406</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67359619143271</v>
+        <v>4.673670212420327</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686672325459038</v>
+        <v>4.686746369269657</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702666985953012</v>
+        <v>4.702756251318035</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705782777672652</v>
+        <v>4.705842091753068</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694857092567699</v>
+        <v>4.694917551319351</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.66490121220027</v>
+        <v>4.664966662089304</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649677525290071</v>
+        <v>4.649688482626038</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641451165057606</v>
+        <v>4.641476287045034</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636262307893886</v>
+        <v>4.636277619318578</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634077281508503</v>
+        <v>4.634113355439964</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637406256185238</v>
+        <v>4.63741558548392</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634390596095246</v>
+        <v>4.634370710519168</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627443337277058</v>
+        <v>4.627382995905593</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62369222361461</v>
+        <v>4.623627839854271</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599054072584001</v>
+        <v>4.598990728153504</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579257567693807</v>
+        <v>4.579123121134869</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560295580315382</v>
+        <v>4.560078890188345</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522046273422818</v>
+        <v>4.521725201250476</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518842919069789</v>
+        <v>4.518386105756634</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531548237518736</v>
+        <v>4.531041678369686</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.55039201375366</v>
+        <v>4.549875019981715</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582767950175429</v>
+        <v>4.582186702291263</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.60108737628941</v>
+        <v>4.600342647383654</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673484018943933</v>
+        <v>4.672630034105199</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.70897989631057</v>
+        <v>4.708074297909557</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775798156101363</v>
+        <v>4.77494099843371</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812086893805286</v>
+        <v>4.811584263234142</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809862811727189</v>
+        <v>4.809369708642353</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819070355325569</v>
+        <v>4.818576418257579</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862253183503444</v>
+        <v>4.862202332297056</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855037718428507</v>
+        <v>4.855007519898155</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853420766881301</v>
+        <v>4.85364868459678</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830462462258145</v>
+        <v>4.830624315579007</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838421994150176</v>
+        <v>4.838636062454847</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891734825775365</v>
+        <v>4.892115593973013</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918041245071505</v>
+        <v>4.918266518392503</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927266946329362</v>
+        <v>4.927495802114937</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917367021435004</v>
+        <v>4.917591538891176</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898136256793526</v>
+        <v>4.898316266083313</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896661370484582</v>
+        <v>4.8969643464574</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897531967893042</v>
+        <v>4.897958875585974</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.8951231676468</v>
+        <v>4.895689404706685</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879652928870575</v>
+        <v>4.880235309913572</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856137632819761</v>
+        <v>4.85662651683514</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829854260434959</v>
+        <v>4.830318613705049</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820563136964852</v>
+        <v>4.821005461110918</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790399519619315</v>
+        <v>4.790766831419985</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.76246371830128</v>
+        <v>4.762837863607031</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.754161082569833</v>
+        <v>4.751946773057718</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756070390823817</v>
+        <v>4.756744839991761</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749351625754665</v>
+        <v>4.750997761831359</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746783366000766</v>
+        <v>4.750513399807955</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.749898471482578</v>
+        <v>4.755189054811616</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.751714646796709</v>
+        <v>4.759038663573635</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.754771157079228</v>
+        <v>4.766032656984724</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.761361447439354</v>
+        <v>4.772175066299832</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.75931715062923</v>
+        <v>4.769870474435316</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.753434924081958</v>
+        <v>4.763122388512472</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.73840884947211</v>
+        <v>4.746594064431817</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.726029704351049</v>
+        <v>4.735993795987901</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.726152688549943</v>
+        <v>4.736134226291687</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.739074832150575</v>
+        <v>4.743700159494207</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.738960076408929</v>
+        <v>4.744664531974359</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.741526044559249</v>
+        <v>4.742726345379941</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.73565068798594</v>
+        <v>4.729672499321643</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.72167422113746</v>
+        <v>4.717834049434108</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.694505389633514</v>
+        <v>4.692141685024607</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.655872121761959</v>
+        <v>4.656282915796599</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.612562565041443</v>
+        <v>4.596208972220294</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.534758397774175</v>
+        <v>4.522301750560466</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.472037576596928</v>
+        <v>4.461343940402478</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.401364474041877</v>
+        <v>4.386963846842344</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.405114655033812</v>
+        <v>4.362522162527467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-12_22-53-26
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.736134226291687</v>
+        <v>4.736146674309882</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.743700159494207</v>
+        <v>4.743693612971123</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.744664531974359</v>
+        <v>4.744808372426592</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.742726345379941</v>
+        <v>4.742743332095513</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.729672499321643</v>
+        <v>4.729685998976733</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.717834049434108</v>
+        <v>4.717845139842323</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.692141685024607</v>
+        <v>4.692151244415032</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.656282915796599</v>
+        <v>4.656291662196194</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.596208972220294</v>
+        <v>4.596220289775951</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.522301750560466</v>
+        <v>4.522313556246317</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.461343940402478</v>
+        <v>4.461356166628916</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.386963846842344</v>
+        <v>4.386978525847038</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.362522162527467</v>
+        <v>4.362548151414771</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-13_20-36-14
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712815451894418</v>
+        <v>4.712809422156198</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711761684032766</v>
+        <v>4.711789725320361</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720296966913136</v>
+        <v>4.720331432404078</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707167560271485</v>
+        <v>4.707238693627814</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694516913889694</v>
+        <v>4.694588858035329</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678593837271508</v>
+        <v>4.678666406549942</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673603521850532</v>
+        <v>4.673676284673077</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686679657769708</v>
+        <v>4.68675244375999</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702675823115986</v>
+        <v>4.702763577041796</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705788649085278</v>
+        <v>4.705846960080545</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694863077503729</v>
+        <v>4.694922513385115</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664907691650231</v>
+        <v>4.664972033366698</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649678599989306</v>
+        <v>4.64968939187056</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641453644194279</v>
+        <v>4.64147835660126</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636263823750038</v>
+        <v>4.636278875837768</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634080851388779</v>
+        <v>4.63411631729825</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637407172847457</v>
+        <v>4.637416357998048</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634388624902878</v>
+        <v>4.634369081113125</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627437365596385</v>
+        <v>4.627378041854969</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623685850436147</v>
+        <v>4.623622555350057</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599047800858815</v>
+        <v>4.59898553038667</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.5792442359582</v>
+        <v>4.579112109137959</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560274083632661</v>
+        <v>4.560061151590147</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522014433054569</v>
+        <v>4.521698906368823</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518797625568149</v>
+        <v>4.51834868598619</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531498028055736</v>
+        <v>4.531000167465328</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550340783256731</v>
+        <v>4.549832640932888</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582710373017675</v>
+        <v>4.582139035940178</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.601013692742358</v>
+        <v>4.600281486772579</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673399516783292</v>
+        <v>4.672559909714613</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708890284902091</v>
+        <v>4.707999937355223</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.775713439333154</v>
+        <v>4.774870514424375</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.812037208706917</v>
+        <v>4.811542939813489</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809814090255863</v>
+        <v>4.809329146795003</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.819021578982753</v>
+        <v>4.818535760422375</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862248186941123</v>
+        <v>4.86219812162434</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855034769191637</v>
+        <v>4.855005001375276</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853443315593273</v>
+        <v>4.8536674038447</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830478506370953</v>
+        <v>4.830637577587231</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838443197992547</v>
+        <v>4.838653618956249</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891772511994999</v>
+        <v>4.892146851679149</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918063593378326</v>
+        <v>4.918284959320428</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927289642193898</v>
+        <v>4.927514544032356</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917389238893117</v>
+        <v>4.917609973489297</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898154078609513</v>
+        <v>4.898331037438184</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896691321848115</v>
+        <v>4.896989253129279</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897574123238543</v>
+        <v>4.897994017752512</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895179109891517</v>
+        <v>4.89573598760243</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879710476913154</v>
+        <v>4.88028321031338</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856185974963108</v>
+        <v>4.856666694363773</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829900237783347</v>
+        <v>4.830356714617736</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820606947669816</v>
+        <v>4.821041740067836</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790435962539044</v>
+        <v>4.790796896001693</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762500782814383</v>
+        <v>4.762868542770804</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.754197440404718</v>
+        <v>4.751978215255185</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756133074235156</v>
+        <v>4.75679564049568</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749394881612178</v>
+        <v>4.751030270517985</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746801526595442</v>
+        <v>4.750520787115691</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.749878959711014</v>
+        <v>4.755162306377241</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.75163756843123</v>
+        <v>4.758963014858904</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.754647169508059</v>
+        <v>4.765915055786175</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.761204699847987</v>
+        <v>4.772033468727547</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.759149888648505</v>
+        <v>4.769725294726793</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.753294229852388</v>
+        <v>4.763013070153518</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.738317306033551</v>
+        <v>4.746543046990782</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.725993588380712</v>
+        <v>4.735994217173577</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.724438281359872</v>
+        <v>4.734434844521067</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.736865319219486</v>
+        <v>4.74165395061813</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.736709183800174</v>
+        <v>4.742593066054408</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.738350562272</v>
+        <v>4.73962661783389</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.731622701271938</v>
+        <v>4.726526205484124</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.717668588268012</v>
+        <v>4.714292172994847</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.69049193634855</v>
+        <v>4.688549987359072</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.6523524979354</v>
+        <v>4.652988232590324</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.609819561432195</v>
+        <v>4.594112370147608</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.533838164862619</v>
+        <v>4.521633295592107</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.472883719271158</v>
+        <v>4.462299051391306</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.405794486576152</v>
+        <v>4.391779464396471</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.406282489688509</v>
+        <v>4.370350516181676</v>
       </c>
     </row>
     <row r="121" spans="1:2">
@@ -1354,7 +1354,7 @@
         <v>46402</v>
       </c>
       <c r="B121">
-        <v>4.389101802064383</v>
+        <v>4.385080426426143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-14_20-33-49
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712809422156198</v>
+        <v>4.712814855230546</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711789725320361</v>
+        <v>4.711764459791539</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720331432404078</v>
+        <v>4.720300377105684</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707238693627814</v>
+        <v>4.707174599758295</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694588858035329</v>
+        <v>4.694524033591122</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678666406549942</v>
+        <v>4.678601018838553</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673676284673077</v>
+        <v>4.673610722438372</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68675244375999</v>
+        <v>4.68668686029552</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702763577041796</v>
+        <v>4.702684504390717</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705846960080545</v>
+        <v>4.705794417055547</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694922513385115</v>
+        <v>4.694868956951511</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664972033366698</v>
+        <v>4.664914056803559</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64968939187056</v>
+        <v>4.649679657885559</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64147835660126</v>
+        <v>4.641456081291172</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636278875837768</v>
+        <v>4.636265312856521</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.63411631729825</v>
+        <v>4.634084358595198</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637416357998048</v>
+        <v>4.637408074823274</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634369081113125</v>
+        <v>4.634386689025769</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627378041854969</v>
+        <v>4.627431498818609</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623622555350057</v>
+        <v>4.623679589523932</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59898553038667</v>
+        <v>4.599041639916377</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579112109137959</v>
+        <v>4.579231144034479</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560061151590147</v>
+        <v>4.560252975693226</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521698906368823</v>
+        <v>4.521983166017675</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.51834868598619</v>
+        <v>4.518753145888986</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531000167465328</v>
+        <v>4.531448717224751</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.549832640932888</v>
+        <v>4.550290466818294</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582139035940178</v>
+        <v>4.582653818756863</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600281486772579</v>
+        <v>4.600941299549605</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.672559909714613</v>
+        <v>4.673316496314477</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.707999937355223</v>
+        <v>4.708802245215725</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.774870514424375</v>
+        <v>4.775630186783939</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.811542939813489</v>
+        <v>4.811988384025145</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809329146795003</v>
+        <v>4.809766207832275</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818535760422375</v>
+        <v>4.818973636726311</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86219812162434</v>
+        <v>4.862243270463164</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855005001375276</v>
+        <v>4.855031863343399</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.8536674038447</v>
+        <v>4.853465469730587</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830637577587231</v>
+        <v>4.830494263014311</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838653618956249</v>
+        <v>4.838464025390882</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.892146851679149</v>
+        <v>4.891809535441361</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918284959320428</v>
+        <v>4.918085537543922</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927514544032356</v>
+        <v>4.927311929320361</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917609973489297</v>
+        <v>4.917411066516673</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898331037438184</v>
+        <v>4.898171585865719</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896989253129279</v>
+        <v>4.89672075409726</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897994017752512</v>
+        <v>4.897615558122583</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.89573598760243</v>
+        <v>4.895234089889127</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.88028321031338</v>
+        <v>4.879767032737919</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856666694363773</v>
+        <v>4.856233476523716</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.830356714617736</v>
+        <v>4.829945402633699</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.821041740067836</v>
+        <v>4.820649981045802</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790796896001693</v>
+        <v>4.79047174566028</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762868542770804</v>
+        <v>4.762537188471093</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751978215255185</v>
+        <v>4.754233164661352</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75679564049568</v>
+        <v>4.756194729676271</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.751030270517985</v>
+        <v>4.749437483724672</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750520787115691</v>
+        <v>4.746819478512339</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.755162306377241</v>
+        <v>4.749859901048112</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.758963014858904</v>
+        <v>4.75156189967698</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.765915055786175</v>
+        <v>4.754525336749484</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.772033468727547</v>
+        <v>4.761050598603981</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.769725294726793</v>
+        <v>4.758985267020122</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.763013070153518</v>
+        <v>4.753155513197289</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.746543046990782</v>
+        <v>4.738226717418911</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.735994217173577</v>
+        <v>4.725957435420121</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.734434844521067</v>
+        <v>4.723182913870765</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.74165395061813</v>
+        <v>4.735198357988943</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.742593066054408</v>
+        <v>4.735044455780072</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.73962661783389</v>
+        <v>4.735957282302588</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.726526205484124</v>
+        <v>4.728586619705002</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.714292172994847</v>
+        <v>4.714575329032809</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.688549987359072</v>
+        <v>4.687481802487414</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.652988232590324</v>
+        <v>4.649933676489814</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.594112370147608</v>
+        <v>4.60830025631717</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.521633295592107</v>
+        <v>4.534216006419382</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.462299051391306</v>
+        <v>4.475178494384362</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.391779464396471</v>
+        <v>4.41167197909257</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.370350516181676</v>
+        <v>4.41091716651755</v>
       </c>
     </row>
     <row r="121" spans="1:2">
@@ -1354,7 +1354,7 @@
         <v>46402</v>
       </c>
       <c r="B121">
-        <v>4.385080426426143</v>
+        <v>4.402890543151923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-10-16_20-33-43
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712814269033649</v>
+        <v>4.712813693030702</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711767186648236</v>
+        <v>4.711769865883791</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720303727537225</v>
+        <v>4.72030701976484</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.707181515629655</v>
+        <v>4.707188311112884</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694531028273309</v>
+        <v>4.694537901200106</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678608074299672</v>
+        <v>4.678615006947107</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673617796614664</v>
+        <v>4.673624747678891</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686693936451657</v>
+        <v>4.686700889534536</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702693033865096</v>
+        <v>4.702701415485345</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705800084292882</v>
+        <v>4.70580565341291</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694874733675253</v>
+        <v>4.694880410343435</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664920310657695</v>
+        <v>4.664926456106187</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649680699362919</v>
+        <v>4.649681724794124</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641458477406712</v>
+        <v>4.641460833564159</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636266775915233</v>
+        <v>4.636268213603722</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.634087804763289</v>
+        <v>4.634091191472189</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637408962458743</v>
+        <v>4.637409836089285</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634384787524121</v>
+        <v>4.634382919491163</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627425734204615</v>
+        <v>4.627420069109787</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623673437937958</v>
+        <v>4.623667392839967</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599035586848247</v>
+        <v>4.599029638846872</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579218285514024</v>
+        <v>4.579205654214396</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560232246057661</v>
+        <v>4.560211884656659</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.521952456981483</v>
+        <v>4.52192229115653</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.518709458318451</v>
+        <v>4.518666541907528</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.531400281145297</v>
+        <v>4.531352696774569</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.550241040227914</v>
+        <v>4.550192480121452</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.582598260420736</v>
+        <v>4.582543671975492</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.600870163145766</v>
+        <v>4.600800251118386</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.673234918948378</v>
+        <v>4.673154747422894</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.708715736305664</v>
+        <v>4.708630718634591</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.77554836086458</v>
+        <v>4.775467925260077</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81194039762962</v>
+        <v>4.811893228141504</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.809719143000642</v>
+        <v>4.809672875029392</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.818926507386143</v>
+        <v>4.818880170501069</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862238432179074</v>
+        <v>4.862233670256672</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855028999969074</v>
+        <v>4.855026178178032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.853487239555461</v>
+        <v>4.853508634977461</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830509739839844</v>
+        <v>4.830524944230213</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.838484486272402</v>
+        <v>4.838504590218641</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.891845913438749</v>
+        <v>4.891881662713141</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.918107088410379</v>
+        <v>4.918128256436143</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.927333818626405</v>
+        <v>4.927355320645154</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.917432514456398</v>
+        <v>4.917453592514326</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.898188786795695</v>
+        <v>4.898205689348869</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.896749680586435</v>
+        <v>4.896778114216764</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.897656290817004</v>
+        <v>4.897696338982396</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.895288132209057</v>
+        <v>4.895341260592915</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.879822621752089</v>
+        <v>4.879877268503938</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856280159218379</v>
+        <v>4.856326044022818</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.829989776319476</v>
+        <v>4.830033379434274</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.820692257586662</v>
+        <v>4.820733797072549</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790506886701917</v>
+        <v>4.790541402755333</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.762572952601124</v>
+        <v>4.762608091934513</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.754268271651696</v>
+        <v>4.754302777136148</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.756255382002257</v>
+        <v>4.756315055281371</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749479446388115</v>
+        <v>4.749520783500385</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746837224436111</v>
+        <v>4.746854767049443</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.749841281084373</v>
+        <v>4.749823085985447</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.751487602816994</v>
+        <v>4.751414641448768</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.75440560394531</v>
+        <v>4.754287918055818</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.760899078557426</v>
+        <v>4.760750076634515</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.758823225765995</v>
+        <v>4.758663706635581</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.753018735903698</v>
+        <v>4.752883860606923</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.738137075578239</v>
+        <v>4.738048372177793</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.725921262896995</v>
+        <v>4.725885087122546</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.721868808083594</v>
+        <v>4.719555268701544</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.733482649872634</v>
+        <v>4.73055613121416</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.733331069147111</v>
+        <v>4.730240790860523</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.733543252278158</v>
+        <v>4.729698746456426</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.725796247327517</v>
+        <v>4.721386580898946</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.711533428233603</v>
+        <v>4.70663144298843</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.684550229805575</v>
+        <v>4.679409826861813</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.64759617530635</v>
+        <v>4.642572445784761</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1314,7 +1314,7 @@
         <v>46367</v>
       </c>
       <c r="B116">
-        <v>4.606839807646892</v>
+        <v>4.60205706062155</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1322,7 +1322,7 @@
         <v>46374</v>
       </c>
       <c r="B117">
-        <v>4.534579712648684</v>
+        <v>4.530546562254849</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1330,7 +1330,7 @@
         <v>46381</v>
       </c>
       <c r="B118">
-        <v>4.47725964164563</v>
+        <v>4.473569677896519</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1338,7 +1338,7 @@
         <v>46388</v>
       </c>
       <c r="B119">
-        <v>4.41670142098546</v>
+        <v>4.413498830657172</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1346,7 +1346,7 @@
         <v>46395</v>
       </c>
       <c r="B120">
-        <v>4.414472838004132</v>
+        <v>4.405612714439896</v>
       </c>
     </row>
     <row r="121" spans="1:2">
@@ -1354,7 +1354,7 @@
         <v>46402</v>
       </c>
       <c r="B121">
-        <v>4.40759014553282</v>
+        <v>4.38366760974258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>